<commit_message>
feat: add category and cabinet management features with custom context menu UI and services
</commit_message>
<xml_diff>
--- a/Resources/CabinetTemplate.xlsx
+++ b/Resources/CabinetTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Ace\excel-ct-tools\Resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Ace\ExcelAddInCTtools\bin\Debug\net48\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6957B36F-FE30-4D41-BD66-8E481910297B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{609ADBB7-9E68-4855-B2B1-13A60C7D0A78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="15" windowWidth="19440" windowHeight="15000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="项目信息" sheetId="1" r:id="rId1"/>
@@ -494,7 +494,7 @@
     <numFmt numFmtId="181" formatCode="&quot;图号:&quot;@"/>
     <numFmt numFmtId="182" formatCode="0.00_);[Red]\(0.00\)"/>
   </numFmts>
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -585,12 +585,6 @@
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -1173,11 +1167,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="220">
+  <cellXfs count="217">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1363,7 +1357,7 @@
     <xf numFmtId="49" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="14" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="8" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1452,7 +1446,7 @@
     <xf numFmtId="5" fontId="8" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1495,10 +1489,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="19" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="18" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="177" fontId="8" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1534,7 +1525,7 @@
     <xf numFmtId="177" fontId="5" fillId="6" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="1" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1564,16 +1555,16 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="21" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="4" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1693,7 +1684,7 @@
     <xf numFmtId="177" fontId="5" fillId="14" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1702,26 +1693,20 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1730,10 +1715,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
     <xf numFmtId="1" fontId="8" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1763,12 +1748,43 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1810,37 +1826,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2271,23 +2256,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="214" t="str">
+      <c r="A1" s="195" t="str">
         <f>T(B22)</f>
         <v>扬州华科</v>
       </c>
-      <c r="B1" s="214"/>
-      <c r="C1" s="214"/>
-      <c r="D1" s="214"/>
+      <c r="B1" s="195"/>
+      <c r="C1" s="195"/>
+      <c r="D1" s="195"/>
       <c r="H1" s="1"/>
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="215" t="str">
+      <c r="A2" s="196" t="str">
         <f>T(B23)</f>
         <v/>
       </c>
-      <c r="B2" s="215"/>
-      <c r="C2" s="215"/>
-      <c r="D2" s="215"/>
+      <c r="B2" s="196"/>
+      <c r="C2" s="196"/>
+      <c r="D2" s="196"/>
       <c r="H2" s="1"/>
     </row>
     <row r="3" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
@@ -2301,14 +2286,14 @@
       <c r="H3" s="5"/>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="216" t="s">
+      <c r="A4" s="197" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="216"/>
-      <c r="C4" s="216"/>
-      <c r="D4" s="216"/>
-      <c r="E4" s="216"/>
-      <c r="F4" s="216"/>
+      <c r="B4" s="197"/>
+      <c r="C4" s="197"/>
+      <c r="D4" s="197"/>
+      <c r="E4" s="197"/>
+      <c r="F4" s="197"/>
       <c r="G4" s="4"/>
       <c r="H4" s="5"/>
     </row>
@@ -2316,9 +2301,9 @@
       <c r="A5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="217"/>
-      <c r="C5" s="218"/>
-      <c r="D5" s="219"/>
+      <c r="B5" s="198"/>
+      <c r="C5" s="199"/>
+      <c r="D5" s="200"/>
       <c r="E5" s="6" t="s">
         <v>7</v>
       </c>
@@ -2332,9 +2317,9 @@
       <c r="A6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="183"/>
-      <c r="C6" s="197"/>
-      <c r="D6" s="184"/>
+      <c r="B6" s="180"/>
+      <c r="C6" s="194"/>
+      <c r="D6" s="181"/>
       <c r="E6" s="6" t="s">
         <v>10</v>
       </c>
@@ -2346,9 +2331,9 @@
       <c r="A7" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="217"/>
-      <c r="C7" s="218"/>
-      <c r="D7" s="219"/>
+      <c r="B7" s="198"/>
+      <c r="C7" s="199"/>
+      <c r="D7" s="200"/>
       <c r="E7" s="9"/>
       <c r="F7" s="10"/>
       <c r="G7" s="4"/>
@@ -2358,11 +2343,11 @@
       <c r="A8" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="B8" s="183" t="s">
+      <c r="B8" s="180" t="s">
         <v>94</v>
       </c>
-      <c r="C8" s="197"/>
-      <c r="D8" s="184"/>
+      <c r="C8" s="194"/>
+      <c r="D8" s="181"/>
       <c r="E8" s="11"/>
       <c r="F8" s="12"/>
       <c r="G8" s="4"/>
@@ -2372,9 +2357,9 @@
       <c r="A9" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="183"/>
-      <c r="C9" s="197"/>
-      <c r="D9" s="184"/>
+      <c r="B9" s="180"/>
+      <c r="C9" s="194"/>
+      <c r="D9" s="181"/>
       <c r="E9" s="11"/>
       <c r="F9" s="12"/>
       <c r="G9" s="4"/>
@@ -2384,9 +2369,9 @@
       <c r="A10" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="183"/>
-      <c r="C10" s="197"/>
-      <c r="D10" s="184"/>
+      <c r="B10" s="180"/>
+      <c r="C10" s="194"/>
+      <c r="D10" s="181"/>
       <c r="E10" s="11"/>
       <c r="F10" s="12"/>
       <c r="G10" s="4"/>
@@ -2396,9 +2381,9 @@
       <c r="A11" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="183"/>
-      <c r="C11" s="197"/>
-      <c r="D11" s="184"/>
+      <c r="B11" s="180"/>
+      <c r="C11" s="194"/>
+      <c r="D11" s="181"/>
       <c r="E11" s="11"/>
       <c r="F11" s="12"/>
       <c r="G11" s="4"/>
@@ -2408,21 +2393,21 @@
       <c r="A12" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="183"/>
-      <c r="C12" s="197"/>
-      <c r="D12" s="184"/>
+      <c r="B12" s="180"/>
+      <c r="C12" s="194"/>
+      <c r="D12" s="181"/>
       <c r="E12" s="11"/>
       <c r="F12" s="12"/>
       <c r="G12" s="4"/>
       <c r="H12" s="5"/>
     </row>
     <row r="13" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="211" t="s">
+      <c r="A13" s="201" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="212"/>
-      <c r="C13" s="212"/>
-      <c r="D13" s="213"/>
+      <c r="B13" s="202"/>
+      <c r="C13" s="202"/>
+      <c r="D13" s="203"/>
       <c r="E13" s="11"/>
       <c r="F13" s="12"/>
       <c r="G13" s="4"/>
@@ -2432,9 +2417,9 @@
       <c r="A14" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="183"/>
-      <c r="C14" s="197"/>
-      <c r="D14" s="184"/>
+      <c r="B14" s="180"/>
+      <c r="C14" s="194"/>
+      <c r="D14" s="181"/>
       <c r="E14" s="11"/>
       <c r="F14" s="12"/>
       <c r="G14" s="4"/>
@@ -2444,9 +2429,9 @@
       <c r="A15" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="183"/>
-      <c r="C15" s="197"/>
-      <c r="D15" s="184"/>
+      <c r="B15" s="180"/>
+      <c r="C15" s="194"/>
+      <c r="D15" s="181"/>
       <c r="E15" s="11"/>
       <c r="F15" s="12"/>
       <c r="G15" s="4"/>
@@ -2456,9 +2441,9 @@
       <c r="A16" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="183"/>
-      <c r="C16" s="197"/>
-      <c r="D16" s="184"/>
+      <c r="B16" s="180"/>
+      <c r="C16" s="194"/>
+      <c r="D16" s="181"/>
       <c r="E16" s="11"/>
       <c r="F16" s="12"/>
       <c r="G16" s="4"/>
@@ -2468,9 +2453,9 @@
       <c r="A17" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="183"/>
-      <c r="C17" s="197"/>
-      <c r="D17" s="184"/>
+      <c r="B17" s="180"/>
+      <c r="C17" s="194"/>
+      <c r="D17" s="181"/>
       <c r="E17" s="11"/>
       <c r="F17" s="12"/>
       <c r="G17" s="4"/>
@@ -2480,9 +2465,9 @@
       <c r="A18" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="183"/>
-      <c r="C18" s="197"/>
-      <c r="D18" s="184"/>
+      <c r="B18" s="180"/>
+      <c r="C18" s="194"/>
+      <c r="D18" s="181"/>
       <c r="E18" s="11"/>
       <c r="F18" s="12"/>
       <c r="G18" s="4"/>
@@ -2492,9 +2477,9 @@
       <c r="A19" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="183"/>
-      <c r="C19" s="197"/>
-      <c r="D19" s="184"/>
+      <c r="B19" s="180"/>
+      <c r="C19" s="194"/>
+      <c r="D19" s="181"/>
       <c r="E19" s="11"/>
       <c r="F19" s="12"/>
       <c r="G19" s="4"/>
@@ -2504,21 +2489,21 @@
       <c r="A20" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="183"/>
-      <c r="C20" s="197"/>
-      <c r="D20" s="184"/>
+      <c r="B20" s="180"/>
+      <c r="C20" s="194"/>
+      <c r="D20" s="181"/>
       <c r="E20" s="11"/>
       <c r="F20" s="12"/>
       <c r="G20" s="4"/>
       <c r="H20" s="5"/>
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A21" s="211" t="s">
+      <c r="A21" s="201" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="212"/>
-      <c r="C21" s="212"/>
-      <c r="D21" s="213"/>
+      <c r="B21" s="202"/>
+      <c r="C21" s="202"/>
+      <c r="D21" s="203"/>
       <c r="E21" s="11"/>
       <c r="F21" s="12"/>
       <c r="G21" s="4"/>
@@ -2528,11 +2513,11 @@
       <c r="A22" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B22" s="183" t="s">
+      <c r="B22" s="180" t="s">
         <v>95</v>
       </c>
-      <c r="C22" s="197"/>
-      <c r="D22" s="184"/>
+      <c r="C22" s="194"/>
+      <c r="D22" s="181"/>
       <c r="E22" s="11"/>
       <c r="F22" s="12"/>
       <c r="G22" s="4"/>
@@ -2542,9 +2527,9 @@
       <c r="A23" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="183"/>
-      <c r="C23" s="197"/>
-      <c r="D23" s="184"/>
+      <c r="B23" s="180"/>
+      <c r="C23" s="194"/>
+      <c r="D23" s="181"/>
       <c r="E23" s="11"/>
       <c r="F23" s="12"/>
       <c r="G23" s="4"/>
@@ -2554,9 +2539,9 @@
       <c r="A24" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B24" s="183"/>
-      <c r="C24" s="197"/>
-      <c r="D24" s="184"/>
+      <c r="B24" s="180"/>
+      <c r="C24" s="194"/>
+      <c r="D24" s="181"/>
       <c r="E24" s="11"/>
       <c r="F24" s="12"/>
       <c r="G24" s="4"/>
@@ -2566,9 +2551,9 @@
       <c r="A25" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B25" s="183"/>
-      <c r="C25" s="197"/>
-      <c r="D25" s="184"/>
+      <c r="B25" s="180"/>
+      <c r="C25" s="194"/>
+      <c r="D25" s="181"/>
       <c r="E25" s="11"/>
       <c r="F25" s="12"/>
       <c r="G25" s="4"/>
@@ -2578,21 +2563,21 @@
       <c r="A26" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B26" s="183"/>
-      <c r="C26" s="197"/>
-      <c r="D26" s="184"/>
+      <c r="B26" s="180"/>
+      <c r="C26" s="194"/>
+      <c r="D26" s="181"/>
       <c r="E26" s="11"/>
       <c r="F26" s="12"/>
       <c r="G26" s="4"/>
       <c r="H26" s="5"/>
     </row>
     <row r="27" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A27" s="198" t="s">
+      <c r="A27" s="204" t="s">
         <v>28</v>
       </c>
-      <c r="B27" s="199"/>
-      <c r="C27" s="199"/>
-      <c r="D27" s="200"/>
+      <c r="B27" s="205"/>
+      <c r="C27" s="205"/>
+      <c r="D27" s="206"/>
       <c r="E27" s="13"/>
       <c r="F27" s="14"/>
       <c r="G27" s="4"/>
@@ -2625,13 +2610,13 @@
       </c>
     </row>
     <row r="29" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A29" s="108">
+      <c r="A29" s="107">
         <f t="shared" ref="A29:A56" si="0">ROW()-ROW(A$28)</f>
         <v>1</v>
       </c>
-      <c r="B29" s="21" t="e">
-        <f ca="1">MID(CELL("filename",folderTablefde937420be6433383ffe23c6ac3a25c),SEARCH({"xlsx]",".xls]"},CELL("filename",folderTablefde937420be6433383ffe23c6ac3a25c))+5,31)</f>
-        <v>#NAME?</v>
+      <c r="B29" s="21" t="str">
+        <f ca="1">MID(CELL("filename",分类1!$A$1),FIND("]",CELL("filename",分类1!$A$1))+1,31)</f>
+        <v>分类1</v>
       </c>
       <c r="C29" s="22">
         <f ca="1">IF(H29="箱变",分类1!F35,分类1!F31*IF(分类1!F35="",1,分类1!F35))</f>
@@ -3033,33 +3018,33 @@
       <c r="B56" s="47" t="s">
         <v>40</v>
       </c>
-      <c r="C56" s="201" t="str">
+      <c r="C56" s="207" t="str">
         <f ca="1">TEXT(SUBSTITUTE(IF(D55="","",IF(MOD(D55,1)=0,TEXT(INT(D55),"[DBNum2][$-804]G/通用格式元整"),(TEXT(INT(D55),"[DBNum2][$-804]G/通用格式元")&amp;TEXT((INT(D55*10)-INT(D55)*10),"[DBNum2][$-804]G/通用格式角")&amp;TEXT((INT(D55*100)-INT(D55*10)*10),"[DBNum2][$-804]G/通用格式分")))),"零角","零"),)</f>
         <v>零元整</v>
       </c>
-      <c r="D56" s="202"/>
+      <c r="D56" s="208"/>
       <c r="E56" s="4"/>
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
       <c r="H56" s="5"/>
     </row>
     <row r="57" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A57" s="203" t="s">
+      <c r="A57" s="209" t="s">
         <v>41</v>
       </c>
-      <c r="B57" s="205"/>
-      <c r="C57" s="206"/>
-      <c r="D57" s="207"/>
+      <c r="B57" s="211"/>
+      <c r="C57" s="212"/>
+      <c r="D57" s="213"/>
       <c r="E57" s="4"/>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
       <c r="H57" s="5"/>
     </row>
     <row r="58" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A58" s="204"/>
-      <c r="B58" s="208"/>
-      <c r="C58" s="209"/>
-      <c r="D58" s="210"/>
+      <c r="A58" s="210"/>
+      <c r="B58" s="214"/>
+      <c r="C58" s="215"/>
+      <c r="D58" s="216"/>
       <c r="E58" s="4"/>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
@@ -3074,6 +3059,24 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="C56:D56"/>
+    <mergeCell ref="A57:A58"/>
+    <mergeCell ref="B57:D58"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B23:D23"/>
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
@@ -3086,24 +3089,6 @@
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="C56:D56"/>
-    <mergeCell ref="A57:A58"/>
-    <mergeCell ref="B57:D58"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations disablePrompts="1" count="1">
@@ -3154,62 +3139,62 @@
       <c r="I1" s="58"/>
     </row>
     <row r="2" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="175" t="str">
-        <f>T(项目信息!B22)</f>
+      <c r="A2" s="174" t="str">
+        <f ca="1">T(INDIRECT("项目信息!B22"))</f>
         <v>扬州华科</v>
       </c>
-      <c r="B2" s="175"/>
-      <c r="C2" s="175"/>
-      <c r="D2" s="175"/>
-      <c r="E2" s="175"/>
-      <c r="F2" s="175"/>
-      <c r="G2" s="175"/>
-      <c r="H2" s="175"/>
-      <c r="I2" s="175"/>
+      <c r="B2" s="174"/>
+      <c r="C2" s="174"/>
+      <c r="D2" s="174"/>
+      <c r="E2" s="174"/>
+      <c r="F2" s="174"/>
+      <c r="G2" s="174"/>
+      <c r="H2" s="174"/>
+      <c r="I2" s="174"/>
     </row>
     <row r="3" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="176" t="str">
-        <f>T(项目信息!B23)</f>
-        <v/>
-      </c>
-      <c r="B3" s="176"/>
-      <c r="C3" s="176"/>
-      <c r="D3" s="176"/>
-      <c r="E3" s="176"/>
-      <c r="F3" s="176"/>
-      <c r="G3" s="176"/>
-      <c r="H3" s="176"/>
-      <c r="I3" s="177"/>
+      <c r="A3" s="174" t="str">
+        <f ca="1">T(INDIRECT("项目信息!B23"))</f>
+        <v/>
+      </c>
+      <c r="B3" s="174"/>
+      <c r="C3" s="174"/>
+      <c r="D3" s="174"/>
+      <c r="E3" s="174"/>
+      <c r="F3" s="174"/>
+      <c r="G3" s="174"/>
+      <c r="H3" s="174"/>
+      <c r="I3" s="174"/>
     </row>
     <row r="4" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="178" t="s">
+      <c r="A4" s="175" t="s">
         <v>42</v>
       </c>
-      <c r="B4" s="179"/>
-      <c r="C4" s="179"/>
-      <c r="D4" s="179"/>
-      <c r="E4" s="179"/>
-      <c r="F4" s="179"/>
-      <c r="G4" s="179"/>
-      <c r="H4" s="179"/>
-      <c r="I4" s="179"/>
+      <c r="B4" s="176"/>
+      <c r="C4" s="176"/>
+      <c r="D4" s="176"/>
+      <c r="E4" s="176"/>
+      <c r="F4" s="176"/>
+      <c r="G4" s="176"/>
+      <c r="H4" s="176"/>
+      <c r="I4" s="176"/>
     </row>
     <row r="5" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="180" t="str">
-        <f>CONCATENATE("项目名称:",项目信息!B5)</f>
+      <c r="A5" s="177" t="str" cm="1">
+        <f t="array" aca="1" ref="A5" ca="1">CONCATENATE("项目名称:",INDIRECT("项目信息!$B$5"))</f>
         <v>项目名称:</v>
       </c>
-      <c r="B5" s="181"/>
-      <c r="C5" s="181"/>
-      <c r="D5" s="181"/>
-      <c r="E5" s="181"/>
-      <c r="F5" s="181"/>
-      <c r="G5" s="182"/>
-      <c r="H5" s="183" t="str">
-        <f>CONCATENATE("报价序号:",项目信息!B7)</f>
+      <c r="B5" s="178"/>
+      <c r="C5" s="178"/>
+      <c r="D5" s="178"/>
+      <c r="E5" s="178"/>
+      <c r="F5" s="178"/>
+      <c r="G5" s="179"/>
+      <c r="H5" s="180" t="str">
+        <f ca="1">CONCATENATE("报价序号:", INDIRECT("'项目信息'!B7"))</f>
         <v>报价序号:</v>
       </c>
-      <c r="I5" s="184"/>
+      <c r="I5" s="181"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
@@ -3288,11 +3273,11 @@
       <c r="F7" s="68">
         <v>1</v>
       </c>
-      <c r="G7" s="110"/>
-      <c r="H7" s="110"/>
+      <c r="G7" s="109"/>
+      <c r="H7" s="109"/>
       <c r="I7" s="69"/>
-      <c r="J7" s="116"/>
-      <c r="K7" s="118"/>
+      <c r="J7" s="115"/>
+      <c r="K7" s="117"/>
       <c r="L7" s="70"/>
       <c r="M7" s="71"/>
       <c r="N7" s="72"/>
@@ -3310,11 +3295,11 @@
       <c r="D8" s="67"/>
       <c r="E8" s="68"/>
       <c r="F8" s="68"/>
-      <c r="G8" s="110"/>
-      <c r="H8" s="110"/>
+      <c r="G8" s="109"/>
+      <c r="H8" s="109"/>
       <c r="I8" s="69"/>
-      <c r="J8" s="116"/>
-      <c r="K8" s="118"/>
+      <c r="J8" s="115"/>
+      <c r="K8" s="117"/>
       <c r="L8" s="70"/>
       <c r="M8" s="71"/>
       <c r="N8" s="72"/>
@@ -3332,11 +3317,11 @@
       <c r="D9" s="76"/>
       <c r="E9" s="77"/>
       <c r="F9" s="68"/>
-      <c r="G9" s="110"/>
-      <c r="H9" s="110"/>
+      <c r="G9" s="109"/>
+      <c r="H9" s="109"/>
       <c r="I9" s="69"/>
-      <c r="J9" s="116"/>
-      <c r="K9" s="118"/>
+      <c r="J9" s="115"/>
+      <c r="K9" s="117"/>
       <c r="L9" s="78"/>
       <c r="M9" s="71"/>
       <c r="N9" s="72"/>
@@ -3354,11 +3339,11 @@
       <c r="D10" s="67"/>
       <c r="E10" s="68"/>
       <c r="F10" s="68"/>
-      <c r="G10" s="110"/>
-      <c r="H10" s="110"/>
+      <c r="G10" s="109"/>
+      <c r="H10" s="109"/>
       <c r="I10" s="69"/>
-      <c r="J10" s="116"/>
-      <c r="K10" s="118"/>
+      <c r="J10" s="115"/>
+      <c r="K10" s="117"/>
       <c r="L10" s="70"/>
       <c r="M10" s="71"/>
       <c r="N10" s="72"/>
@@ -3376,11 +3361,11 @@
       <c r="D11" s="67"/>
       <c r="E11" s="68"/>
       <c r="F11" s="68"/>
-      <c r="G11" s="110"/>
-      <c r="H11" s="110"/>
+      <c r="G11" s="109"/>
+      <c r="H11" s="109"/>
       <c r="I11" s="69"/>
-      <c r="J11" s="116"/>
-      <c r="K11" s="118"/>
+      <c r="J11" s="115"/>
+      <c r="K11" s="117"/>
       <c r="L11" s="70"/>
       <c r="M11" s="71"/>
       <c r="N11" s="72"/>
@@ -3398,11 +3383,11 @@
       <c r="D12" s="67"/>
       <c r="E12" s="68"/>
       <c r="F12" s="68"/>
-      <c r="G12" s="110"/>
-      <c r="H12" s="110"/>
+      <c r="G12" s="109"/>
+      <c r="H12" s="109"/>
       <c r="I12" s="69"/>
-      <c r="J12" s="116"/>
-      <c r="K12" s="118"/>
+      <c r="J12" s="115"/>
+      <c r="K12" s="117"/>
       <c r="L12" s="70"/>
       <c r="M12" s="71"/>
       <c r="N12" s="72"/>
@@ -3420,11 +3405,11 @@
       <c r="D13" s="67"/>
       <c r="E13" s="68"/>
       <c r="F13" s="68"/>
-      <c r="G13" s="110"/>
-      <c r="H13" s="110"/>
+      <c r="G13" s="109"/>
+      <c r="H13" s="109"/>
       <c r="I13" s="69"/>
-      <c r="J13" s="116"/>
-      <c r="K13" s="118"/>
+      <c r="J13" s="115"/>
+      <c r="K13" s="117"/>
       <c r="L13" s="70"/>
       <c r="M13" s="71"/>
       <c r="N13" s="72"/>
@@ -3442,11 +3427,11 @@
       <c r="D14" s="67"/>
       <c r="E14" s="68"/>
       <c r="F14" s="68"/>
-      <c r="G14" s="110"/>
-      <c r="H14" s="110"/>
+      <c r="G14" s="109"/>
+      <c r="H14" s="109"/>
       <c r="I14" s="69"/>
-      <c r="J14" s="116"/>
-      <c r="K14" s="118"/>
+      <c r="J14" s="115"/>
+      <c r="K14" s="117"/>
       <c r="L14" s="70"/>
       <c r="M14" s="71"/>
       <c r="N14" s="72"/>
@@ -3464,11 +3449,11 @@
       <c r="D15" s="67"/>
       <c r="E15" s="68"/>
       <c r="F15" s="68"/>
-      <c r="G15" s="110"/>
-      <c r="H15" s="110"/>
+      <c r="G15" s="109"/>
+      <c r="H15" s="109"/>
       <c r="I15" s="69"/>
-      <c r="J15" s="116"/>
-      <c r="K15" s="118"/>
+      <c r="J15" s="115"/>
+      <c r="K15" s="117"/>
       <c r="L15" s="70"/>
       <c r="M15" s="71"/>
       <c r="N15" s="72"/>
@@ -3486,11 +3471,11 @@
       <c r="D16" s="67"/>
       <c r="E16" s="68"/>
       <c r="F16" s="68"/>
-      <c r="G16" s="110"/>
-      <c r="H16" s="110"/>
+      <c r="G16" s="109"/>
+      <c r="H16" s="109"/>
       <c r="I16" s="69"/>
-      <c r="J16" s="116"/>
-      <c r="K16" s="118"/>
+      <c r="J16" s="115"/>
+      <c r="K16" s="117"/>
       <c r="L16" s="70"/>
       <c r="M16" s="71"/>
       <c r="N16" s="72"/>
@@ -3508,11 +3493,11 @@
       <c r="D17" s="67"/>
       <c r="E17" s="68"/>
       <c r="F17" s="79"/>
-      <c r="G17" s="110"/>
-      <c r="H17" s="110"/>
+      <c r="G17" s="109"/>
+      <c r="H17" s="109"/>
       <c r="I17" s="69"/>
-      <c r="J17" s="116"/>
-      <c r="K17" s="118"/>
+      <c r="J17" s="115"/>
+      <c r="K17" s="117"/>
       <c r="L17" s="70"/>
       <c r="M17" s="71"/>
       <c r="N17" s="72"/>
@@ -3530,11 +3515,11 @@
       <c r="D18" s="67"/>
       <c r="E18" s="68"/>
       <c r="F18" s="79"/>
-      <c r="G18" s="110"/>
-      <c r="H18" s="110"/>
+      <c r="G18" s="109"/>
+      <c r="H18" s="109"/>
       <c r="I18" s="69"/>
-      <c r="J18" s="116"/>
-      <c r="K18" s="118"/>
+      <c r="J18" s="115"/>
+      <c r="K18" s="117"/>
       <c r="L18" s="70"/>
       <c r="M18" s="71"/>
       <c r="N18" s="72"/>
@@ -3552,11 +3537,11 @@
       <c r="D19" s="67"/>
       <c r="E19" s="68"/>
       <c r="F19" s="79"/>
-      <c r="G19" s="110"/>
-      <c r="H19" s="110"/>
+      <c r="G19" s="109"/>
+      <c r="H19" s="109"/>
       <c r="I19" s="69"/>
-      <c r="J19" s="116"/>
-      <c r="K19" s="118"/>
+      <c r="J19" s="115"/>
+      <c r="K19" s="117"/>
       <c r="L19" s="70"/>
       <c r="M19" s="71"/>
       <c r="N19" s="72"/>
@@ -3574,11 +3559,11 @@
       <c r="D20" s="67"/>
       <c r="E20" s="68"/>
       <c r="F20" s="79"/>
-      <c r="G20" s="110"/>
-      <c r="H20" s="110"/>
+      <c r="G20" s="109"/>
+      <c r="H20" s="109"/>
       <c r="I20" s="69"/>
-      <c r="J20" s="116"/>
-      <c r="K20" s="118"/>
+      <c r="J20" s="115"/>
+      <c r="K20" s="117"/>
       <c r="L20" s="70"/>
       <c r="M20" s="71"/>
       <c r="N20" s="72"/>
@@ -3596,11 +3581,11 @@
       <c r="D21" s="67"/>
       <c r="E21" s="68"/>
       <c r="F21" s="79"/>
-      <c r="G21" s="110"/>
-      <c r="H21" s="110"/>
+      <c r="G21" s="109"/>
+      <c r="H21" s="109"/>
       <c r="I21" s="69"/>
-      <c r="J21" s="116"/>
-      <c r="K21" s="118"/>
+      <c r="J21" s="115"/>
+      <c r="K21" s="117"/>
       <c r="L21" s="70"/>
       <c r="M21" s="71"/>
       <c r="N21" s="72"/>
@@ -3618,11 +3603,11 @@
       <c r="D22" s="67"/>
       <c r="E22" s="68"/>
       <c r="F22" s="68"/>
-      <c r="G22" s="110"/>
-      <c r="H22" s="110"/>
+      <c r="G22" s="109"/>
+      <c r="H22" s="109"/>
       <c r="I22" s="69"/>
-      <c r="J22" s="116"/>
-      <c r="K22" s="118"/>
+      <c r="J22" s="115"/>
+      <c r="K22" s="117"/>
       <c r="L22" s="70"/>
       <c r="M22" s="71"/>
       <c r="N22" s="72"/>
@@ -3640,11 +3625,11 @@
       <c r="D23" s="67"/>
       <c r="E23" s="68"/>
       <c r="F23" s="68"/>
-      <c r="G23" s="110"/>
-      <c r="H23" s="110"/>
+      <c r="G23" s="109"/>
+      <c r="H23" s="109"/>
       <c r="I23" s="69"/>
-      <c r="J23" s="116"/>
-      <c r="K23" s="118"/>
+      <c r="J23" s="115"/>
+      <c r="K23" s="117"/>
       <c r="L23" s="70"/>
       <c r="M23" s="71"/>
       <c r="N23" s="72"/>
@@ -3662,11 +3647,11 @@
       <c r="D24" s="67"/>
       <c r="E24" s="77"/>
       <c r="F24" s="77"/>
-      <c r="G24" s="111"/>
-      <c r="H24" s="111"/>
+      <c r="G24" s="110"/>
+      <c r="H24" s="110"/>
       <c r="I24" s="69"/>
-      <c r="J24" s="116"/>
-      <c r="K24" s="118"/>
+      <c r="J24" s="115"/>
+      <c r="K24" s="117"/>
       <c r="L24" s="70"/>
       <c r="M24" s="71"/>
       <c r="N24" s="72"/>
@@ -3684,11 +3669,11 @@
       <c r="D25" s="67"/>
       <c r="E25" s="77"/>
       <c r="F25" s="80"/>
-      <c r="G25" s="111"/>
-      <c r="H25" s="111"/>
+      <c r="G25" s="110"/>
+      <c r="H25" s="110"/>
       <c r="I25" s="69"/>
-      <c r="J25" s="116"/>
-      <c r="K25" s="118"/>
+      <c r="J25" s="115"/>
+      <c r="K25" s="117"/>
       <c r="L25" s="70"/>
       <c r="M25" s="71"/>
       <c r="N25" s="72"/>
@@ -3706,11 +3691,11 @@
       <c r="D26" s="67"/>
       <c r="E26" s="77"/>
       <c r="F26" s="80"/>
-      <c r="G26" s="111"/>
-      <c r="H26" s="111"/>
+      <c r="G26" s="110"/>
+      <c r="H26" s="110"/>
       <c r="I26" s="69"/>
-      <c r="J26" s="116"/>
-      <c r="K26" s="118"/>
+      <c r="J26" s="115"/>
+      <c r="K26" s="117"/>
       <c r="L26" s="70"/>
       <c r="M26" s="71"/>
       <c r="N26" s="72"/>
@@ -3728,11 +3713,11 @@
       <c r="D27" s="67"/>
       <c r="E27" s="68"/>
       <c r="F27" s="68"/>
-      <c r="G27" s="110"/>
-      <c r="H27" s="110"/>
+      <c r="G27" s="109"/>
+      <c r="H27" s="109"/>
       <c r="I27" s="69"/>
-      <c r="J27" s="116"/>
-      <c r="K27" s="118"/>
+      <c r="J27" s="115"/>
+      <c r="K27" s="117"/>
       <c r="L27" s="70"/>
       <c r="M27" s="71"/>
       <c r="N27" s="72"/>
@@ -3750,11 +3735,11 @@
       <c r="D28" s="67"/>
       <c r="E28" s="68"/>
       <c r="F28" s="68"/>
-      <c r="G28" s="110"/>
-      <c r="H28" s="110"/>
+      <c r="G28" s="109"/>
+      <c r="H28" s="109"/>
       <c r="I28" s="69"/>
-      <c r="J28" s="116"/>
-      <c r="K28" s="118"/>
+      <c r="J28" s="115"/>
+      <c r="K28" s="117"/>
       <c r="L28" s="70"/>
       <c r="M28" s="71"/>
       <c r="N28" s="72"/>
@@ -3772,11 +3757,11 @@
       <c r="D29" s="67"/>
       <c r="E29" s="68"/>
       <c r="F29" s="68"/>
-      <c r="G29" s="110"/>
-      <c r="H29" s="110"/>
+      <c r="G29" s="109"/>
+      <c r="H29" s="109"/>
       <c r="I29" s="69"/>
-      <c r="J29" s="116"/>
-      <c r="K29" s="118"/>
+      <c r="J29" s="115"/>
+      <c r="K29" s="117"/>
       <c r="L29" s="70"/>
       <c r="M29" s="71"/>
       <c r="N29" s="72"/>
@@ -3794,11 +3779,11 @@
       <c r="D30" s="67"/>
       <c r="E30" s="68"/>
       <c r="F30" s="68"/>
-      <c r="G30" s="110"/>
-      <c r="H30" s="110"/>
+      <c r="G30" s="109"/>
+      <c r="H30" s="109"/>
       <c r="I30" s="69"/>
-      <c r="J30" s="116"/>
-      <c r="K30" s="118"/>
+      <c r="J30" s="115"/>
+      <c r="K30" s="117"/>
       <c r="L30" s="70"/>
       <c r="M30" s="71"/>
       <c r="N30" s="72"/>
@@ -3823,17 +3808,17 @@
         <f>SUM(F6:INDEX(F:F,ROW()-1))</f>
         <v>1</v>
       </c>
-      <c r="G31" s="112"/>
-      <c r="H31" s="113">
+      <c r="G31" s="111"/>
+      <c r="H31" s="112">
         <f>ROUND(SUM(H6:INDEX(H:H,ROW()-1)),2)</f>
         <v>0</v>
       </c>
       <c r="I31" s="84"/>
-      <c r="J31" s="116">
+      <c r="J31" s="115">
         <f>ROUND(SUM(J6:INDEX(J:J,ROW()-1)),2)</f>
         <v>0</v>
       </c>
-      <c r="K31" s="118">
+      <c r="K31" s="117">
         <f>ROUND(SUM(K6:INDEX(K:K,ROW()-1)),2)</f>
         <v>0</v>
       </c>
@@ -3860,19 +3845,19 @@
       <c r="F32" s="83">
         <v>1</v>
       </c>
-      <c r="G32" s="113">
+      <c r="G32" s="112">
         <v>0</v>
       </c>
-      <c r="H32" s="113">
+      <c r="H32" s="112">
         <f>ROUND(F32*G32,2)</f>
         <v>0</v>
       </c>
       <c r="I32" s="87"/>
-      <c r="J32" s="116">
+      <c r="J32" s="115">
         <f>ROUND(H32,2)</f>
         <v>0</v>
       </c>
-      <c r="K32" s="118"/>
+      <c r="K32" s="117"/>
       <c r="L32" s="70"/>
       <c r="M32" s="88"/>
       <c r="N32" s="89"/>
@@ -3896,19 +3881,19 @@
       <c r="F33" s="83">
         <v>1</v>
       </c>
-      <c r="G33" s="113">
+      <c r="G33" s="112">
         <v>0</v>
       </c>
-      <c r="H33" s="113">
+      <c r="H33" s="112">
         <f>ROUND(F33*G33,2)</f>
         <v>0</v>
       </c>
       <c r="I33" s="87"/>
-      <c r="J33" s="116">
+      <c r="J33" s="115">
         <f>ROUND(H33,2)</f>
         <v>0</v>
       </c>
-      <c r="K33" s="118"/>
+      <c r="K33" s="117"/>
       <c r="L33" s="70"/>
       <c r="M33" s="88"/>
       <c r="N33" s="89"/>
@@ -3932,19 +3917,19 @@
       <c r="F34" s="83">
         <v>1</v>
       </c>
-      <c r="G34" s="113">
+      <c r="G34" s="112">
         <v>0</v>
       </c>
-      <c r="H34" s="113">
+      <c r="H34" s="112">
         <f>ROUND(F34*G34,2)</f>
         <v>0</v>
       </c>
       <c r="I34" s="91"/>
-      <c r="J34" s="116">
+      <c r="J34" s="115">
         <f>ROUND(H34,2)</f>
         <v>0</v>
       </c>
-      <c r="K34" s="118"/>
+      <c r="K34" s="117"/>
       <c r="L34" s="70"/>
       <c r="M34" s="88"/>
       <c r="N34" s="89"/>
@@ -3960,30 +3945,30 @@
       <c r="B35" s="92" t="s">
         <v>60</v>
       </c>
-      <c r="C35" s="185" t="str">
+      <c r="C35" s="182" t="str">
         <f ca="1">TEXT(SUBSTITUTE(IF(H35="","",IF(MOD(H35,1)=0,TEXT(INT(H35),"[DBNum2][$-804]G/通用格式元整"),(TEXT(INT(H35),"[DBNum2][$-804]G/通用格式元")&amp;TEXT((INT(H35*10)-INT(H35)*10),"[DBNum2][$-804]G/通用格式角")&amp;TEXT((INT(H35*100)-INT(H35*10)*10),"[DBNum2][$-804]G/通用格式分")))),"零角","零"),)</f>
         <v>零元整</v>
       </c>
-      <c r="D35" s="186"/>
+      <c r="D35" s="183"/>
       <c r="E35" s="93"/>
       <c r="F35" s="94" t="str">
-        <f ca="1">IF(项目信息!H29="箱变",1,"")</f>
-        <v/>
-      </c>
-      <c r="G35" s="114">
+        <f ca="1">IF(INDIRECT("'项目信息'!H29")="箱变", 1, "")</f>
+        <v/>
+      </c>
+      <c r="G35" s="113">
         <f>ROUND(SUM(H31:H34),2)</f>
         <v>0</v>
       </c>
-      <c r="H35" s="114">
+      <c r="H35" s="113">
         <f ca="1">ROUND(IF(F35="",1,F35)*G35,2)</f>
         <v>0</v>
       </c>
       <c r="I35" s="95"/>
-      <c r="J35" s="117">
+      <c r="J35" s="116">
         <f ca="1">ROUND(IF(F35="",1,F35)*SUM(J31:J34),2)</f>
         <v>0</v>
       </c>
-      <c r="K35" s="119">
+      <c r="K35" s="118">
         <f ca="1">ROUND(IF(F35="",1,F35)*SUM(K31:K34),2)</f>
         <v>0</v>
       </c>
@@ -3998,19 +3983,19 @@
       <c r="Q35" s="101"/>
     </row>
     <row r="36" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A36" s="187" t="s">
+      <c r="A36" s="184" t="s">
         <v>61</v>
       </c>
-      <c r="B36" s="189"/>
-      <c r="C36" s="190"/>
-      <c r="D36" s="190"/>
-      <c r="E36" s="190"/>
-      <c r="F36" s="190"/>
-      <c r="G36" s="191"/>
-      <c r="H36" s="191"/>
-      <c r="I36" s="192"/>
-      <c r="J36" s="115"/>
-      <c r="K36" s="115"/>
+      <c r="B36" s="186"/>
+      <c r="C36" s="187"/>
+      <c r="D36" s="187"/>
+      <c r="E36" s="187"/>
+      <c r="F36" s="187"/>
+      <c r="G36" s="188"/>
+      <c r="H36" s="188"/>
+      <c r="I36" s="189"/>
+      <c r="J36" s="114"/>
+      <c r="K36" s="114"/>
       <c r="L36" s="4"/>
       <c r="M36" s="4"/>
       <c r="N36" s="4"/>
@@ -4019,17 +4004,17 @@
       <c r="Q36" s="4"/>
     </row>
     <row r="37" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A37" s="188"/>
-      <c r="B37" s="193"/>
-      <c r="C37" s="193"/>
-      <c r="D37" s="193"/>
-      <c r="E37" s="193"/>
-      <c r="F37" s="193"/>
-      <c r="G37" s="194"/>
-      <c r="H37" s="194"/>
-      <c r="I37" s="195"/>
-      <c r="J37" s="115"/>
-      <c r="K37" s="115"/>
+      <c r="A37" s="185"/>
+      <c r="B37" s="190"/>
+      <c r="C37" s="190"/>
+      <c r="D37" s="190"/>
+      <c r="E37" s="190"/>
+      <c r="F37" s="190"/>
+      <c r="G37" s="191"/>
+      <c r="H37" s="191"/>
+      <c r="I37" s="192"/>
+      <c r="J37" s="114"/>
+      <c r="K37" s="114"/>
       <c r="L37" s="4"/>
       <c r="M37" s="4"/>
       <c r="N37" s="4"/>
@@ -4044,11 +4029,11 @@
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
-      <c r="G38" s="115"/>
-      <c r="H38" s="115"/>
+      <c r="G38" s="114"/>
+      <c r="H38" s="114"/>
       <c r="I38" s="104"/>
-      <c r="J38" s="115"/>
-      <c r="K38" s="115"/>
+      <c r="J38" s="114"/>
+      <c r="K38" s="114"/>
       <c r="L38" s="4"/>
       <c r="M38" s="4"/>
       <c r="N38" s="4"/>
@@ -4063,11 +4048,11 @@
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
       <c r="F39" s="4"/>
-      <c r="G39" s="115"/>
-      <c r="H39" s="115"/>
+      <c r="G39" s="114"/>
+      <c r="H39" s="114"/>
       <c r="I39" s="4"/>
-      <c r="J39" s="115"/>
-      <c r="K39" s="115"/>
+      <c r="J39" s="114"/>
+      <c r="K39" s="114"/>
       <c r="L39" s="4"/>
       <c r="M39" s="4"/>
       <c r="N39" s="4"/>
@@ -4076,18 +4061,18 @@
       <c r="Q39" s="4"/>
     </row>
     <row r="40" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A40" s="105" t="str">
-        <f>CONCATENATE("报价人：",项目信息!B8)</f>
+      <c r="A40" s="105"/>
+      <c r="B40" s="172" t="str" cm="1">
+        <f t="array" aca="1" ref="B40" ca="1">CONCATENATE("报价人：", INDIRECT("项目信息!$B$8"))</f>
         <v>报价人：李四</v>
       </c>
-      <c r="B40" s="54"/>
       <c r="C40" s="54"/>
       <c r="D40" s="106"/>
       <c r="E40" s="106"/>
       <c r="F40" s="106"/>
       <c r="G40" s="104"/>
-      <c r="H40" s="107">
-        <f>项目信息!B9</f>
+      <c r="H40" s="158" cm="1">
+        <f t="array" aca="1" ref="H40" ca="1">INDIRECT("项目信息!$B$9")</f>
         <v>0</v>
       </c>
       <c r="I40" s="4"/>
@@ -4101,89 +4086,89 @@
       <c r="Q40" s="4"/>
     </row>
     <row r="41" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A41" s="175" t="str">
-        <f>T(项目信息!$B$22)</f>
+      <c r="A41" s="174" t="str">
+        <f ca="1">T(INDIRECT("项目信息!B22"))</f>
         <v>扬州华科</v>
       </c>
-      <c r="B41" s="175"/>
-      <c r="C41" s="175"/>
-      <c r="D41" s="175"/>
-      <c r="E41" s="175"/>
-      <c r="F41" s="175"/>
-      <c r="G41" s="175"/>
-      <c r="H41" s="175"/>
-      <c r="I41" s="175"/>
+      <c r="B41" s="174"/>
+      <c r="C41" s="174"/>
+      <c r="D41" s="174"/>
+      <c r="E41" s="174"/>
+      <c r="F41" s="174"/>
+      <c r="G41" s="174"/>
+      <c r="H41" s="174"/>
+      <c r="I41" s="174"/>
       <c r="Q41" s="1"/>
       <c r="R41" s="1"/>
     </row>
     <row r="42" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A42" s="176" t="str">
-        <f>T(项目信息!$B$23)</f>
-        <v/>
-      </c>
-      <c r="B42" s="176"/>
-      <c r="C42" s="176"/>
-      <c r="D42" s="176"/>
-      <c r="E42" s="176"/>
-      <c r="F42" s="176"/>
-      <c r="G42" s="176"/>
-      <c r="H42" s="176"/>
-      <c r="I42" s="176"/>
+      <c r="A42" s="174" t="str">
+        <f ca="1">T(INDIRECT("项目信息!B23"))</f>
+        <v/>
+      </c>
+      <c r="B42" s="174"/>
+      <c r="C42" s="174"/>
+      <c r="D42" s="174"/>
+      <c r="E42" s="174"/>
+      <c r="F42" s="174"/>
+      <c r="G42" s="174"/>
+      <c r="H42" s="174"/>
+      <c r="I42" s="174"/>
       <c r="Q42" s="1"/>
       <c r="R42" s="1"/>
     </row>
     <row r="43" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A43" s="196" t="s">
+      <c r="A43" s="193" t="s">
         <v>64</v>
       </c>
-      <c r="B43" s="196"/>
-      <c r="C43" s="196"/>
-      <c r="D43" s="196"/>
-      <c r="E43" s="196"/>
-      <c r="F43" s="196"/>
-      <c r="G43" s="196"/>
-      <c r="H43" s="196"/>
-      <c r="I43" s="196"/>
+      <c r="B43" s="193"/>
+      <c r="C43" s="193"/>
+      <c r="D43" s="193"/>
+      <c r="E43" s="193"/>
+      <c r="F43" s="193"/>
+      <c r="G43" s="193"/>
+      <c r="H43" s="193"/>
+      <c r="I43" s="193"/>
       <c r="Q43" s="1"/>
       <c r="R43" s="1"/>
     </row>
-    <row r="44" spans="1:21" s="128" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A44" s="120" t="s">
+    <row r="44" spans="1:21" s="127" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A44" s="119" t="s">
         <v>92</v>
       </c>
-      <c r="B44" s="121" t="s">
+      <c r="B44" s="120" t="s">
         <v>96</v>
       </c>
-      <c r="C44" s="122" t="s">
+      <c r="C44" s="121" t="s">
         <v>65</v>
       </c>
-      <c r="D44" s="174" t="s">
-        <v>8</v>
-      </c>
-      <c r="E44" s="174"/>
-      <c r="F44" s="123" t="s">
+      <c r="D44" s="173" t="s">
+        <v>8</v>
+      </c>
+      <c r="E44" s="173"/>
+      <c r="F44" s="122" t="s">
         <v>66</v>
       </c>
-      <c r="G44" s="174" t="s">
-        <v>8</v>
-      </c>
-      <c r="H44" s="174"/>
-      <c r="I44" s="124" t="s">
-        <v>8</v>
-      </c>
-      <c r="J44" s="125" t="s">
+      <c r="G44" s="173" t="s">
+        <v>8</v>
+      </c>
+      <c r="H44" s="173"/>
+      <c r="I44" s="123" t="s">
+        <v>8</v>
+      </c>
+      <c r="J44" s="124" t="s">
         <v>67</v>
       </c>
-      <c r="K44" s="126" t="s">
-        <v>8</v>
-      </c>
-      <c r="L44" s="125" t="s">
+      <c r="K44" s="125" t="s">
+        <v>8</v>
+      </c>
+      <c r="L44" s="124" t="s">
         <v>68</v>
       </c>
-      <c r="M44" s="126" t="s">
-        <v>8</v>
-      </c>
-      <c r="N44" s="127" t="s">
+      <c r="M44" s="125" t="s">
+        <v>8</v>
+      </c>
+      <c r="N44" s="126" t="s">
         <v>8</v>
       </c>
       <c r="Q44" s="5"/>
@@ -4199,7 +4184,7 @@
       <c r="C45" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="D45" s="129" t="s">
+      <c r="D45" s="128" t="s">
         <v>62</v>
       </c>
       <c r="E45" s="60" t="s">
@@ -4214,43 +4199,43 @@
       <c r="H45" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="I45" s="130" t="s">
+      <c r="I45" s="129" t="s">
         <v>74</v>
       </c>
-      <c r="J45" s="131" t="s">
+      <c r="J45" s="130" t="s">
         <v>75</v>
       </c>
-      <c r="K45" s="131" t="s">
+      <c r="K45" s="130" t="s">
         <v>76</v>
       </c>
-      <c r="L45" s="132" t="s">
+      <c r="L45" s="131" t="s">
         <v>77</v>
       </c>
-      <c r="M45" s="131" t="s">
+      <c r="M45" s="130" t="s">
         <v>78</v>
       </c>
-      <c r="N45" s="132" t="s">
+      <c r="N45" s="131" t="s">
         <v>79</v>
       </c>
-      <c r="O45" s="133" t="s">
+      <c r="O45" s="132" t="s">
         <v>80</v>
       </c>
-      <c r="P45" s="131" t="s">
+      <c r="P45" s="130" t="s">
         <v>81</v>
       </c>
-      <c r="Q45" s="134" t="s">
+      <c r="Q45" s="133" t="s">
         <v>82</v>
       </c>
-      <c r="R45" s="134" t="s">
+      <c r="R45" s="133" t="s">
         <v>83</v>
       </c>
-      <c r="S45" s="134" t="s">
+      <c r="S45" s="133" t="s">
         <v>84</v>
       </c>
-      <c r="T45" s="134" t="s">
+      <c r="T45" s="133" t="s">
         <v>85</v>
       </c>
-      <c r="U45" s="135" t="s">
+      <c r="U45" s="134" t="s">
         <v>8</v>
       </c>
     </row>
@@ -4273,52 +4258,52 @@
         <f t="shared" ref="F46:F65" si="2">IF(AND(B46="",C46=""),"",1)</f>
         <v/>
       </c>
-      <c r="G46" s="109" t="str">
+      <c r="G46" s="108" t="str">
         <f t="shared" ref="G46:G65" si="3">IF(AND(B46="",C46=""),"",ROUND(M46*L46*N46,2))</f>
         <v/>
       </c>
-      <c r="H46" s="109" t="str">
+      <c r="H46" s="108" t="str">
         <f t="shared" ref="H46:H65" si="4">IF(AND(B46="",C46=""),"",ROUND(F46*G46,2))</f>
         <v/>
       </c>
-      <c r="I46" s="136" t="s">
-        <v>8</v>
-      </c>
-      <c r="J46" s="161" t="str">
+      <c r="I46" s="135" t="s">
+        <v>8</v>
+      </c>
+      <c r="J46" s="160" t="str">
         <f t="shared" ref="J46:J65" si="5">IF(AND(B46="",C46=""),"",ROUND(M46*N46,2))</f>
         <v/>
       </c>
-      <c r="K46" s="164" t="str">
+      <c r="K46" s="163" t="str">
         <f t="shared" ref="K46:K65" si="6">IF(AND(B46="",C46=""),"",ROUND(J46*F46,2))</f>
         <v/>
       </c>
-      <c r="L46" s="137" t="str">
+      <c r="L46" s="136" t="str">
         <f t="shared" ref="L46:L65" si="7">IF(AND(B46="",C46=""),"",1)</f>
         <v/>
       </c>
-      <c r="M46" s="167"/>
-      <c r="N46" s="138" t="str">
+      <c r="M46" s="166"/>
+      <c r="N46" s="137" t="str">
         <f t="shared" ref="N46:N65" si="8">IF(AND(B46="",C46=""),"",1)</f>
         <v/>
       </c>
-      <c r="O46" s="139" t="str">
+      <c r="O46" s="138" t="str">
         <f>IF(AND(B46="",C46=""),"",IF(G46&gt;=20000,0.05,IF(G46&gt;=10000,0.1,IF(G46&gt;=5000,0.2,IF(G46&gt;=1000,0.3,IF(G46&gt;=0,0.4,{0}))))))</f>
         <v/>
       </c>
-      <c r="P46" s="170" t="str">
+      <c r="P46" s="169" t="str">
         <f t="shared" ref="P46:P65" si="9">IF(AND(B46="",C46=""),"",ROUND(H46*O46,2))</f>
         <v/>
       </c>
-      <c r="Q46" s="140" t="str">
+      <c r="Q46" s="139" t="str">
         <f t="shared" ref="Q46:Q65" si="10">IF(AND(B46="",C46=""),"","元件")</f>
         <v/>
       </c>
-      <c r="R46" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S46" s="142"/>
-      <c r="T46" s="142"/>
-      <c r="U46" s="143" t="s">
+      <c r="R46" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S46" s="141"/>
+      <c r="T46" s="141"/>
+      <c r="U46" s="142" t="s">
         <v>8</v>
       </c>
     </row>
@@ -4341,52 +4326,52 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G47" s="111" t="str">
+      <c r="G47" s="110" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="H47" s="110" t="str">
+      <c r="H47" s="109" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I47" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="J47" s="162" t="str">
+      <c r="J47" s="161" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="K47" s="165" t="str">
+      <c r="K47" s="164" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="L47" s="137" t="str">
+      <c r="L47" s="136" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="M47" s="168"/>
-      <c r="N47" s="138" t="str">
+      <c r="M47" s="167"/>
+      <c r="N47" s="137" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="O47" s="139" t="str">
+      <c r="O47" s="138" t="str">
         <f>IF(AND(B47="",C47=""),"",IF(G47&gt;=20000,0.05,IF(G47&gt;=10000,0.1,IF(G47&gt;=5000,0.2,IF(G47&gt;=1000,0.3,IF(G47&gt;=0,0.4,{0}))))))</f>
         <v/>
       </c>
-      <c r="P47" s="171" t="str">
+      <c r="P47" s="170" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="Q47" s="140" t="str">
+      <c r="Q47" s="139" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="R47" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S47" s="142"/>
-      <c r="T47" s="142"/>
-      <c r="U47" s="143" t="s">
+      <c r="R47" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S47" s="141"/>
+      <c r="T47" s="141"/>
+      <c r="U47" s="142" t="s">
         <v>8</v>
       </c>
     </row>
@@ -4409,52 +4394,52 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G48" s="110" t="str">
+      <c r="G48" s="109" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="H48" s="110" t="str">
+      <c r="H48" s="109" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I48" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="J48" s="162" t="str">
+      <c r="J48" s="161" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="K48" s="165" t="str">
+      <c r="K48" s="164" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="L48" s="137" t="str">
+      <c r="L48" s="136" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="M48" s="168"/>
-      <c r="N48" s="138" t="str">
+      <c r="M48" s="167"/>
+      <c r="N48" s="137" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="O48" s="139" t="str">
+      <c r="O48" s="138" t="str">
         <f>IF(AND(B48="",C48=""),"",IF(G48&gt;=20000,0.05,IF(G48&gt;=10000,0.1,IF(G48&gt;=5000,0.2,IF(G48&gt;=1000,0.3,IF(G48&gt;=0,0.4,{0}))))))</f>
         <v/>
       </c>
-      <c r="P48" s="171" t="str">
+      <c r="P48" s="170" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="Q48" s="140" t="str">
+      <c r="Q48" s="139" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="R48" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S48" s="142"/>
-      <c r="T48" s="142"/>
-      <c r="U48" s="143" t="s">
+      <c r="R48" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S48" s="141"/>
+      <c r="T48" s="141"/>
+      <c r="U48" s="142" t="s">
         <v>8</v>
       </c>
     </row>
@@ -4477,52 +4462,52 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G49" s="110" t="str">
+      <c r="G49" s="109" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="H49" s="110" t="str">
+      <c r="H49" s="109" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I49" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="J49" s="162" t="str">
+      <c r="J49" s="161" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="K49" s="165" t="str">
+      <c r="K49" s="164" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="L49" s="137" t="str">
+      <c r="L49" s="136" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="M49" s="168"/>
-      <c r="N49" s="138" t="str">
+      <c r="M49" s="167"/>
+      <c r="N49" s="137" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="O49" s="139" t="str">
+      <c r="O49" s="138" t="str">
         <f>IF(AND(B49="",C49=""),"",IF(G49&gt;=20000,0.05,IF(G49&gt;=10000,0.1,IF(G49&gt;=5000,0.2,IF(G49&gt;=1000,0.3,IF(G49&gt;=0,0.4,{0}))))))</f>
         <v/>
       </c>
-      <c r="P49" s="171" t="str">
+      <c r="P49" s="170" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="Q49" s="140" t="str">
+      <c r="Q49" s="139" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="R49" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S49" s="142"/>
-      <c r="T49" s="142"/>
-      <c r="U49" s="143" t="s">
+      <c r="R49" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S49" s="141"/>
+      <c r="T49" s="141"/>
+      <c r="U49" s="142" t="s">
         <v>8</v>
       </c>
     </row>
@@ -4545,52 +4530,52 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G50" s="111" t="str">
+      <c r="G50" s="110" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="H50" s="110" t="str">
+      <c r="H50" s="109" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I50" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="J50" s="162" t="str">
+      <c r="J50" s="161" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="K50" s="165" t="str">
+      <c r="K50" s="164" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="L50" s="137" t="str">
+      <c r="L50" s="136" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="M50" s="168"/>
-      <c r="N50" s="138" t="str">
+      <c r="M50" s="167"/>
+      <c r="N50" s="137" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="O50" s="139" t="str">
+      <c r="O50" s="138" t="str">
         <f>IF(AND(B50="",C50=""),"",IF(G50&gt;=20000,0.05,IF(G50&gt;=10000,0.1,IF(G50&gt;=5000,0.2,IF(G50&gt;=1000,0.3,IF(G50&gt;=0,0.4,{0}))))))</f>
         <v/>
       </c>
-      <c r="P50" s="171" t="str">
+      <c r="P50" s="170" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="Q50" s="140" t="str">
+      <c r="Q50" s="139" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="R50" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S50" s="142"/>
-      <c r="T50" s="142"/>
-      <c r="U50" s="143" t="s">
+      <c r="R50" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S50" s="141"/>
+      <c r="T50" s="141"/>
+      <c r="U50" s="142" t="s">
         <v>8</v>
       </c>
     </row>
@@ -4613,52 +4598,52 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G51" s="111" t="str">
+      <c r="G51" s="110" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="H51" s="110" t="str">
+      <c r="H51" s="109" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I51" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="J51" s="162" t="str">
+      <c r="J51" s="161" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="K51" s="165" t="str">
+      <c r="K51" s="164" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="L51" s="137" t="str">
+      <c r="L51" s="136" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="M51" s="168"/>
-      <c r="N51" s="138" t="str">
+      <c r="M51" s="167"/>
+      <c r="N51" s="137" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="O51" s="139" t="str">
+      <c r="O51" s="138" t="str">
         <f>IF(AND(B51="",C51=""),"",IF(G51&gt;=20000,0.05,IF(G51&gt;=10000,0.1,IF(G51&gt;=5000,0.2,IF(G51&gt;=1000,0.3,IF(G51&gt;=0,0.4,{0}))))))</f>
         <v/>
       </c>
-      <c r="P51" s="171" t="str">
+      <c r="P51" s="170" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="Q51" s="140" t="str">
+      <c r="Q51" s="139" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="R51" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S51" s="142"/>
-      <c r="T51" s="142"/>
-      <c r="U51" s="143" t="s">
+      <c r="R51" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S51" s="141"/>
+      <c r="T51" s="141"/>
+      <c r="U51" s="142" t="s">
         <v>8</v>
       </c>
     </row>
@@ -4681,52 +4666,52 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G52" s="111" t="str">
+      <c r="G52" s="110" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="H52" s="111" t="str">
+      <c r="H52" s="110" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="I52" s="144" t="s">
-        <v>8</v>
-      </c>
-      <c r="J52" s="162" t="str">
+      <c r="I52" s="143" t="s">
+        <v>8</v>
+      </c>
+      <c r="J52" s="161" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="K52" s="165" t="str">
+      <c r="K52" s="164" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="L52" s="137" t="str">
+      <c r="L52" s="136" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="M52" s="168"/>
-      <c r="N52" s="138" t="str">
+      <c r="M52" s="167"/>
+      <c r="N52" s="137" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="O52" s="139" t="str">
+      <c r="O52" s="138" t="str">
         <f>IF(AND(B52="",C52=""),"",IF(G52&gt;=20000,0.05,IF(G52&gt;=10000,0.1,IF(G52&gt;=5000,0.2,IF(G52&gt;=1000,0.3,IF(G52&gt;=0,0.4,{0}))))))</f>
         <v/>
       </c>
-      <c r="P52" s="171" t="str">
+      <c r="P52" s="170" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="Q52" s="140" t="str">
+      <c r="Q52" s="139" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="R52" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S52" s="142"/>
-      <c r="T52" s="142"/>
-      <c r="U52" s="143" t="s">
+      <c r="R52" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S52" s="141"/>
+      <c r="T52" s="141"/>
+      <c r="U52" s="142" t="s">
         <v>8</v>
       </c>
     </row>
@@ -4749,52 +4734,52 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G53" s="111" t="str">
+      <c r="G53" s="110" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="H53" s="111" t="str">
+      <c r="H53" s="110" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="I53" s="144" t="s">
-        <v>8</v>
-      </c>
-      <c r="J53" s="162" t="str">
+      <c r="I53" s="143" t="s">
+        <v>8</v>
+      </c>
+      <c r="J53" s="161" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="K53" s="165" t="str">
+      <c r="K53" s="164" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="L53" s="137" t="str">
+      <c r="L53" s="136" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="M53" s="168"/>
-      <c r="N53" s="138" t="str">
+      <c r="M53" s="167"/>
+      <c r="N53" s="137" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="O53" s="139" t="str">
+      <c r="O53" s="138" t="str">
         <f>IF(AND(B53="",C53=""),"",IF(G53&gt;=20000,0.05,IF(G53&gt;=10000,0.1,IF(G53&gt;=5000,0.2,IF(G53&gt;=1000,0.3,IF(G53&gt;=0,0.4,{0}))))))</f>
         <v/>
       </c>
-      <c r="P53" s="171" t="str">
+      <c r="P53" s="170" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="Q53" s="140" t="str">
+      <c r="Q53" s="139" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="R53" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S53" s="142"/>
-      <c r="T53" s="142"/>
-      <c r="U53" s="143" t="s">
+      <c r="R53" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S53" s="141"/>
+      <c r="T53" s="141"/>
+      <c r="U53" s="142" t="s">
         <v>8</v>
       </c>
     </row>
@@ -4817,52 +4802,52 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G54" s="111" t="str">
+      <c r="G54" s="110" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="H54" s="111" t="str">
+      <c r="H54" s="110" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="I54" s="144" t="s">
-        <v>8</v>
-      </c>
-      <c r="J54" s="162" t="str">
+      <c r="I54" s="143" t="s">
+        <v>8</v>
+      </c>
+      <c r="J54" s="161" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="K54" s="165" t="str">
+      <c r="K54" s="164" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="L54" s="137" t="str">
+      <c r="L54" s="136" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="M54" s="168"/>
-      <c r="N54" s="138" t="str">
+      <c r="M54" s="167"/>
+      <c r="N54" s="137" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="O54" s="139" t="str">
+      <c r="O54" s="138" t="str">
         <f>IF(AND(B54="",C54=""),"",IF(G54&gt;=20000,0.05,IF(G54&gt;=10000,0.1,IF(G54&gt;=5000,0.2,IF(G54&gt;=1000,0.3,IF(G54&gt;=0,0.4,{0}))))))</f>
         <v/>
       </c>
-      <c r="P54" s="171" t="str">
+      <c r="P54" s="170" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="Q54" s="140" t="str">
+      <c r="Q54" s="139" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="R54" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S54" s="142"/>
-      <c r="T54" s="142"/>
-      <c r="U54" s="143" t="s">
+      <c r="R54" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S54" s="141"/>
+      <c r="T54" s="141"/>
+      <c r="U54" s="142" t="s">
         <v>8</v>
       </c>
     </row>
@@ -4885,52 +4870,52 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G55" s="111" t="str">
+      <c r="G55" s="110" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="H55" s="111" t="str">
+      <c r="H55" s="110" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="I55" s="144" t="s">
-        <v>8</v>
-      </c>
-      <c r="J55" s="162" t="str">
+      <c r="I55" s="143" t="s">
+        <v>8</v>
+      </c>
+      <c r="J55" s="161" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="K55" s="165" t="str">
+      <c r="K55" s="164" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="L55" s="137" t="str">
+      <c r="L55" s="136" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="M55" s="168"/>
-      <c r="N55" s="138" t="str">
+      <c r="M55" s="167"/>
+      <c r="N55" s="137" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="O55" s="139" t="str">
+      <c r="O55" s="138" t="str">
         <f>IF(AND(B55="",C55=""),"",IF(G55&gt;=20000,0.05,IF(G55&gt;=10000,0.1,IF(G55&gt;=5000,0.2,IF(G55&gt;=1000,0.3,IF(G55&gt;=0,0.4,{0}))))))</f>
         <v/>
       </c>
-      <c r="P55" s="171" t="str">
+      <c r="P55" s="170" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="Q55" s="140" t="str">
+      <c r="Q55" s="139" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="R55" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S55" s="142"/>
-      <c r="T55" s="142"/>
-      <c r="U55" s="143" t="s">
+      <c r="R55" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S55" s="141"/>
+      <c r="T55" s="141"/>
+      <c r="U55" s="142" t="s">
         <v>8</v>
       </c>
     </row>
@@ -4953,52 +4938,52 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G56" s="111" t="str">
+      <c r="G56" s="110" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="H56" s="111" t="str">
+      <c r="H56" s="110" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="I56" s="144" t="s">
-        <v>8</v>
-      </c>
-      <c r="J56" s="162" t="str">
+      <c r="I56" s="143" t="s">
+        <v>8</v>
+      </c>
+      <c r="J56" s="161" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="K56" s="165" t="str">
+      <c r="K56" s="164" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="L56" s="137" t="str">
+      <c r="L56" s="136" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="M56" s="168"/>
-      <c r="N56" s="138" t="str">
+      <c r="M56" s="167"/>
+      <c r="N56" s="137" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="O56" s="139" t="str">
+      <c r="O56" s="138" t="str">
         <f>IF(AND(B56="",C56=""),"",IF(G56&gt;=20000,0.05,IF(G56&gt;=10000,0.1,IF(G56&gt;=5000,0.2,IF(G56&gt;=1000,0.3,IF(G56&gt;=0,0.4,{0}))))))</f>
         <v/>
       </c>
-      <c r="P56" s="171" t="str">
+      <c r="P56" s="170" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="Q56" s="140" t="str">
+      <c r="Q56" s="139" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="R56" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S56" s="142"/>
-      <c r="T56" s="142"/>
-      <c r="U56" s="143" t="s">
+      <c r="R56" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S56" s="141"/>
+      <c r="T56" s="141"/>
+      <c r="U56" s="142" t="s">
         <v>8</v>
       </c>
     </row>
@@ -5021,52 +5006,52 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G57" s="110" t="str">
+      <c r="G57" s="109" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="H57" s="111" t="str">
+      <c r="H57" s="110" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="I57" s="144" t="s">
-        <v>8</v>
-      </c>
-      <c r="J57" s="162" t="str">
+      <c r="I57" s="143" t="s">
+        <v>8</v>
+      </c>
+      <c r="J57" s="161" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="K57" s="165" t="str">
+      <c r="K57" s="164" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="L57" s="137" t="str">
+      <c r="L57" s="136" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="M57" s="168"/>
-      <c r="N57" s="138" t="str">
+      <c r="M57" s="167"/>
+      <c r="N57" s="137" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="O57" s="139" t="str">
+      <c r="O57" s="138" t="str">
         <f>IF(AND(B57="",C57=""),"",IF(G57&gt;=20000,0.05,IF(G57&gt;=10000,0.1,IF(G57&gt;=5000,0.2,IF(G57&gt;=1000,0.3,IF(G57&gt;=0,0.4,{0}))))))</f>
         <v/>
       </c>
-      <c r="P57" s="171" t="str">
+      <c r="P57" s="170" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="Q57" s="140" t="str">
+      <c r="Q57" s="139" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="R57" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S57" s="142"/>
-      <c r="T57" s="142"/>
-      <c r="U57" s="143" t="s">
+      <c r="R57" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S57" s="141"/>
+      <c r="T57" s="141"/>
+      <c r="U57" s="142" t="s">
         <v>8</v>
       </c>
     </row>
@@ -5089,52 +5074,52 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G58" s="110" t="str">
+      <c r="G58" s="109" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="H58" s="111" t="str">
+      <c r="H58" s="110" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
-      <c r="I58" s="144" t="s">
-        <v>8</v>
-      </c>
-      <c r="J58" s="162" t="str">
+      <c r="I58" s="143" t="s">
+        <v>8</v>
+      </c>
+      <c r="J58" s="161" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="K58" s="165" t="str">
+      <c r="K58" s="164" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="L58" s="137" t="str">
+      <c r="L58" s="136" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="M58" s="168"/>
-      <c r="N58" s="138" t="str">
+      <c r="M58" s="167"/>
+      <c r="N58" s="137" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="O58" s="139" t="str">
+      <c r="O58" s="138" t="str">
         <f>IF(AND(B58="",C58=""),"",IF(G58&gt;=20000,0.05,IF(G58&gt;=10000,0.1,IF(G58&gt;=5000,0.2,IF(G58&gt;=1000,0.3,IF(G58&gt;=0,0.4,{0}))))))</f>
         <v/>
       </c>
-      <c r="P58" s="171" t="str">
+      <c r="P58" s="170" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="Q58" s="140" t="str">
+      <c r="Q58" s="139" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="R58" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S58" s="142"/>
-      <c r="T58" s="142"/>
-      <c r="U58" s="143" t="s">
+      <c r="R58" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S58" s="141"/>
+      <c r="T58" s="141"/>
+      <c r="U58" s="142" t="s">
         <v>8</v>
       </c>
     </row>
@@ -5157,52 +5142,52 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G59" s="110" t="str">
+      <c r="G59" s="109" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="H59" s="110" t="str">
+      <c r="H59" s="109" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I59" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="J59" s="162" t="str">
+      <c r="J59" s="161" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="K59" s="165" t="str">
+      <c r="K59" s="164" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="L59" s="137" t="str">
+      <c r="L59" s="136" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="M59" s="168"/>
-      <c r="N59" s="138" t="str">
+      <c r="M59" s="167"/>
+      <c r="N59" s="137" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="O59" s="139" t="str">
+      <c r="O59" s="138" t="str">
         <f>IF(AND(B59="",C59=""),"",IF(G59&gt;=20000,0.05,IF(G59&gt;=10000,0.1,IF(G59&gt;=5000,0.2,IF(G59&gt;=1000,0.3,IF(G59&gt;=0,0.4,{0}))))))</f>
         <v/>
       </c>
-      <c r="P59" s="171" t="str">
+      <c r="P59" s="170" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="Q59" s="140" t="str">
+      <c r="Q59" s="139" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="R59" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S59" s="142"/>
-      <c r="T59" s="142"/>
-      <c r="U59" s="143" t="s">
+      <c r="R59" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S59" s="141"/>
+      <c r="T59" s="141"/>
+      <c r="U59" s="142" t="s">
         <v>8</v>
       </c>
     </row>
@@ -5225,52 +5210,52 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G60" s="110" t="str">
+      <c r="G60" s="109" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="H60" s="110" t="str">
+      <c r="H60" s="109" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I60" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="J60" s="162" t="str">
+      <c r="J60" s="161" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="K60" s="165" t="str">
+      <c r="K60" s="164" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="L60" s="137" t="str">
+      <c r="L60" s="136" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="M60" s="168"/>
-      <c r="N60" s="138" t="str">
+      <c r="M60" s="167"/>
+      <c r="N60" s="137" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="O60" s="139" t="str">
+      <c r="O60" s="138" t="str">
         <f>IF(AND(B60="",C60=""),"",IF(G60&gt;=20000,0.05,IF(G60&gt;=10000,0.1,IF(G60&gt;=5000,0.2,IF(G60&gt;=1000,0.3,IF(G60&gt;=0,0.4,{0}))))))</f>
         <v/>
       </c>
-      <c r="P60" s="171" t="str">
+      <c r="P60" s="170" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="Q60" s="140" t="str">
+      <c r="Q60" s="139" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="R60" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S60" s="142"/>
-      <c r="T60" s="142"/>
-      <c r="U60" s="143" t="s">
+      <c r="R60" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S60" s="141"/>
+      <c r="T60" s="141"/>
+      <c r="U60" s="142" t="s">
         <v>8</v>
       </c>
     </row>
@@ -5293,52 +5278,52 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G61" s="110" t="str">
+      <c r="G61" s="109" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="H61" s="110" t="str">
+      <c r="H61" s="109" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I61" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="J61" s="162" t="str">
+      <c r="J61" s="161" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="K61" s="165" t="str">
+      <c r="K61" s="164" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="L61" s="137" t="str">
+      <c r="L61" s="136" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="M61" s="168"/>
-      <c r="N61" s="138" t="str">
+      <c r="M61" s="167"/>
+      <c r="N61" s="137" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="O61" s="139" t="str">
+      <c r="O61" s="138" t="str">
         <f>IF(AND(B61="",C61=""),"",IF(G61&gt;=20000,0.05,IF(G61&gt;=10000,0.1,IF(G61&gt;=5000,0.2,IF(G61&gt;=1000,0.3,IF(G61&gt;=0,0.4,{0}))))))</f>
         <v/>
       </c>
-      <c r="P61" s="171" t="str">
+      <c r="P61" s="170" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="Q61" s="140" t="str">
+      <c r="Q61" s="139" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="R61" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S61" s="142"/>
-      <c r="T61" s="142"/>
-      <c r="U61" s="143" t="s">
+      <c r="R61" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S61" s="141"/>
+      <c r="T61" s="141"/>
+      <c r="U61" s="142" t="s">
         <v>8</v>
       </c>
     </row>
@@ -5361,52 +5346,52 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G62" s="110" t="str">
+      <c r="G62" s="109" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="H62" s="110" t="str">
+      <c r="H62" s="109" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I62" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="J62" s="162" t="str">
+      <c r="J62" s="161" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="K62" s="165" t="str">
+      <c r="K62" s="164" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="L62" s="137" t="str">
+      <c r="L62" s="136" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="M62" s="168"/>
-      <c r="N62" s="138" t="str">
+      <c r="M62" s="167"/>
+      <c r="N62" s="137" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="O62" s="139" t="str">
+      <c r="O62" s="138" t="str">
         <f>IF(AND(B62="",C62=""),"",IF(G62&gt;=20000,0.05,IF(G62&gt;=10000,0.1,IF(G62&gt;=5000,0.2,IF(G62&gt;=1000,0.3,IF(G62&gt;=0,0.4,{0}))))))</f>
         <v/>
       </c>
-      <c r="P62" s="171" t="str">
+      <c r="P62" s="170" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="Q62" s="140" t="str">
+      <c r="Q62" s="139" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="R62" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S62" s="142"/>
-      <c r="T62" s="142"/>
-      <c r="U62" s="143" t="s">
+      <c r="R62" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S62" s="141"/>
+      <c r="T62" s="141"/>
+      <c r="U62" s="142" t="s">
         <v>8</v>
       </c>
     </row>
@@ -5429,52 +5414,52 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G63" s="110" t="str">
+      <c r="G63" s="109" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="H63" s="110" t="str">
+      <c r="H63" s="109" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I63" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="J63" s="162" t="str">
+      <c r="J63" s="161" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="K63" s="165" t="str">
+      <c r="K63" s="164" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="L63" s="137" t="str">
+      <c r="L63" s="136" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="M63" s="168"/>
-      <c r="N63" s="138" t="str">
+      <c r="M63" s="167"/>
+      <c r="N63" s="137" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="O63" s="139" t="str">
+      <c r="O63" s="138" t="str">
         <f>IF(AND(B63="",C63=""),"",IF(G63&gt;=20000,0.05,IF(G63&gt;=10000,0.1,IF(G63&gt;=5000,0.2,IF(G63&gt;=1000,0.3,IF(G63&gt;=0,0.4,{0}))))))</f>
         <v/>
       </c>
-      <c r="P63" s="171" t="str">
+      <c r="P63" s="170" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="Q63" s="140" t="str">
+      <c r="Q63" s="139" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="R63" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S63" s="142"/>
-      <c r="T63" s="142"/>
-      <c r="U63" s="143" t="s">
+      <c r="R63" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S63" s="141"/>
+      <c r="T63" s="141"/>
+      <c r="U63" s="142" t="s">
         <v>8</v>
       </c>
     </row>
@@ -5497,52 +5482,52 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G64" s="110" t="str">
+      <c r="G64" s="109" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="H64" s="110" t="str">
+      <c r="H64" s="109" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I64" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="J64" s="162" t="str">
+      <c r="J64" s="161" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="K64" s="165" t="str">
+      <c r="K64" s="164" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="L64" s="137" t="str">
+      <c r="L64" s="136" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="M64" s="168"/>
-      <c r="N64" s="138" t="str">
+      <c r="M64" s="167"/>
+      <c r="N64" s="137" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="O64" s="139" t="str">
+      <c r="O64" s="138" t="str">
         <f>IF(AND(B64="",C64=""),"",IF(G64&gt;=20000,0.05,IF(G64&gt;=10000,0.1,IF(G64&gt;=5000,0.2,IF(G64&gt;=1000,0.3,IF(G64&gt;=0,0.4,{0}))))))</f>
         <v/>
       </c>
-      <c r="P64" s="171" t="str">
+      <c r="P64" s="170" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="Q64" s="140" t="str">
+      <c r="Q64" s="139" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="R64" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S64" s="142"/>
-      <c r="T64" s="142"/>
-      <c r="U64" s="143" t="s">
+      <c r="R64" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S64" s="141"/>
+      <c r="T64" s="141"/>
+      <c r="U64" s="142" t="s">
         <v>8</v>
       </c>
     </row>
@@ -5565,52 +5550,52 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G65" s="110" t="str">
+      <c r="G65" s="109" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="H65" s="110" t="str">
+      <c r="H65" s="109" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
       <c r="I65" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="J65" s="162" t="str">
+      <c r="J65" s="161" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="K65" s="165" t="str">
+      <c r="K65" s="164" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="L65" s="137" t="str">
+      <c r="L65" s="136" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="M65" s="168"/>
-      <c r="N65" s="138" t="str">
+      <c r="M65" s="167"/>
+      <c r="N65" s="137" t="str">
         <f t="shared" si="8"/>
         <v/>
       </c>
-      <c r="O65" s="139" t="str">
+      <c r="O65" s="138" t="str">
         <f>IF(AND(B65="",C65=""),"",IF(G65&gt;=20000,0.05,IF(G65&gt;=10000,0.1,IF(G65&gt;=5000,0.2,IF(G65&gt;=1000,0.3,IF(G65&gt;=0,0.4,{0}))))))</f>
         <v/>
       </c>
-      <c r="P65" s="171" t="str">
+      <c r="P65" s="170" t="str">
         <f t="shared" si="9"/>
         <v/>
       </c>
-      <c r="Q65" s="140" t="str">
+      <c r="Q65" s="139" t="str">
         <f t="shared" si="10"/>
         <v/>
       </c>
-      <c r="R65" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S65" s="142"/>
-      <c r="T65" s="142"/>
-      <c r="U65" s="143" t="s">
+      <c r="R65" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S65" s="141"/>
+      <c r="T65" s="141"/>
+      <c r="U65" s="142" t="s">
         <v>8</v>
       </c>
     </row>
@@ -5619,44 +5604,44 @@
         <f t="shared" si="1"/>
         <v>21</v>
       </c>
-      <c r="B66" s="145" t="s">
+      <c r="B66" s="144" t="s">
         <v>37</v>
       </c>
-      <c r="C66" s="146"/>
+      <c r="C66" s="145"/>
       <c r="D66" s="102"/>
       <c r="E66" s="77"/>
       <c r="F66" s="77"/>
-      <c r="G66" s="111"/>
-      <c r="H66" s="111">
+      <c r="G66" s="110"/>
+      <c r="H66" s="110">
         <f>ROUND(SUM(H45:INDEX(H:H,ROW()-1)),2)</f>
         <v>0</v>
       </c>
       <c r="I66" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="J66" s="162"/>
-      <c r="K66" s="165">
+      <c r="J66" s="161"/>
+      <c r="K66" s="164">
         <f>ROUND(SUM(K45:INDEX(K:K,ROW()-1)),2)</f>
         <v>0</v>
       </c>
-      <c r="L66" s="137"/>
-      <c r="M66" s="168"/>
-      <c r="N66" s="138"/>
-      <c r="O66" s="139"/>
-      <c r="P66" s="171"/>
-      <c r="Q66" s="140"/>
-      <c r="R66" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S66" s="142">
+      <c r="L66" s="136"/>
+      <c r="M66" s="167"/>
+      <c r="N66" s="137"/>
+      <c r="O66" s="138"/>
+      <c r="P66" s="170"/>
+      <c r="Q66" s="139"/>
+      <c r="R66" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S66" s="141">
         <f>ROUND(SUMPRODUCT(F45:INDEX(F:F,ROW()-1),S45:INDEX(S:S,ROW()-1)),2)</f>
         <v>0</v>
       </c>
-      <c r="T66" s="142">
+      <c r="T66" s="141">
         <f>ROUND(SUMPRODUCT(F45:INDEX(F:F,ROW()-1),T45:INDEX(T:T,ROW()-1)),2)</f>
         <v>0</v>
       </c>
-      <c r="U66" s="143" t="s">
+      <c r="U66" s="142" t="s">
         <v>8</v>
       </c>
     </row>
@@ -5665,40 +5650,40 @@
         <f t="shared" si="1"/>
         <v>22</v>
       </c>
-      <c r="B67" s="145" t="s">
+      <c r="B67" s="144" t="s">
         <v>88</v>
       </c>
-      <c r="C67" s="146"/>
+      <c r="C67" s="145"/>
       <c r="D67" s="102"/>
       <c r="E67" s="77"/>
       <c r="F67" s="77"/>
-      <c r="G67" s="111"/>
-      <c r="H67" s="111">
+      <c r="G67" s="110"/>
+      <c r="H67" s="110">
         <f>ROUND(S66*1.18,0)</f>
         <v>0</v>
       </c>
       <c r="I67" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="J67" s="162"/>
-      <c r="K67" s="165">
+      <c r="J67" s="161"/>
+      <c r="K67" s="164">
         <f>H67</f>
         <v>0</v>
       </c>
-      <c r="L67" s="137"/>
-      <c r="M67" s="168"/>
-      <c r="N67" s="138"/>
-      <c r="O67" s="139"/>
-      <c r="P67" s="171"/>
-      <c r="Q67" s="140" t="s">
+      <c r="L67" s="136"/>
+      <c r="M67" s="167"/>
+      <c r="N67" s="137"/>
+      <c r="O67" s="138"/>
+      <c r="P67" s="170"/>
+      <c r="Q67" s="139" t="s">
         <v>89</v>
       </c>
-      <c r="R67" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S67" s="142"/>
-      <c r="T67" s="142"/>
-      <c r="U67" s="143" t="s">
+      <c r="R67" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S67" s="141"/>
+      <c r="T67" s="141"/>
+      <c r="U67" s="142" t="s">
         <v>8</v>
       </c>
     </row>
@@ -5707,35 +5692,35 @@
         <f t="shared" si="1"/>
         <v>23</v>
       </c>
-      <c r="B68" s="145" t="s">
+      <c r="B68" s="144" t="s">
         <v>90</v>
       </c>
-      <c r="C68" s="146"/>
+      <c r="C68" s="145"/>
       <c r="D68" s="102"/>
       <c r="E68" s="77"/>
       <c r="F68" s="77"/>
-      <c r="G68" s="111"/>
-      <c r="H68" s="111">
+      <c r="G68" s="110"/>
+      <c r="H68" s="110">
         <f>ROUND(SUM(H66:H67)*0.1,0)</f>
         <v>0</v>
       </c>
       <c r="I68" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="J68" s="162"/>
-      <c r="K68" s="165"/>
-      <c r="L68" s="137"/>
-      <c r="M68" s="168"/>
-      <c r="N68" s="138"/>
-      <c r="O68" s="139"/>
-      <c r="P68" s="171"/>
-      <c r="Q68" s="140"/>
-      <c r="R68" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S68" s="142"/>
-      <c r="T68" s="142"/>
-      <c r="U68" s="143" t="s">
+      <c r="J68" s="161"/>
+      <c r="K68" s="164"/>
+      <c r="L68" s="136"/>
+      <c r="M68" s="167"/>
+      <c r="N68" s="137"/>
+      <c r="O68" s="138"/>
+      <c r="P68" s="170"/>
+      <c r="Q68" s="139"/>
+      <c r="R68" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S68" s="141"/>
+      <c r="T68" s="141"/>
+      <c r="U68" s="142" t="s">
         <v>8</v>
       </c>
     </row>
@@ -5744,37 +5729,37 @@
         <f t="shared" si="1"/>
         <v>24</v>
       </c>
-      <c r="B69" s="145" t="s">
+      <c r="B69" s="144" t="s">
         <v>91</v>
       </c>
-      <c r="C69" s="146"/>
+      <c r="C69" s="145"/>
       <c r="D69" s="102"/>
       <c r="E69" s="77"/>
       <c r="F69" s="77"/>
-      <c r="G69" s="111"/>
-      <c r="H69" s="111">
+      <c r="G69" s="110"/>
+      <c r="H69" s="110">
         <f>ROUND(SUM(H66:H68)*0.13,0)</f>
         <v>0</v>
       </c>
       <c r="I69" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="J69" s="162"/>
-      <c r="K69" s="165"/>
-      <c r="L69" s="137"/>
-      <c r="M69" s="168"/>
-      <c r="N69" s="138"/>
-      <c r="O69" s="139"/>
-      <c r="P69" s="171"/>
-      <c r="Q69" s="140" t="s">
+      <c r="J69" s="161"/>
+      <c r="K69" s="164"/>
+      <c r="L69" s="136"/>
+      <c r="M69" s="167"/>
+      <c r="N69" s="137"/>
+      <c r="O69" s="138"/>
+      <c r="P69" s="170"/>
+      <c r="Q69" s="139" t="s">
         <v>89</v>
       </c>
-      <c r="R69" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S69" s="142"/>
-      <c r="T69" s="142"/>
-      <c r="U69" s="143" t="s">
+      <c r="R69" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S69" s="141"/>
+      <c r="T69" s="141"/>
+      <c r="U69" s="142" t="s">
         <v>8</v>
       </c>
     </row>
@@ -5786,135 +5771,134 @@
       <c r="B70" s="102" t="s">
         <v>86</v>
       </c>
-      <c r="C70" s="146"/>
+      <c r="C70" s="145"/>
       <c r="D70" s="102"/>
       <c r="E70" s="77"/>
       <c r="F70" s="77"/>
-      <c r="G70" s="111"/>
-      <c r="H70" s="111">
+      <c r="G70" s="110"/>
+      <c r="H70" s="110">
         <f>ROUND(SUM(H66:H69),0)</f>
         <v>0</v>
       </c>
-      <c r="I70" s="147"/>
-      <c r="J70" s="162"/>
-      <c r="K70" s="165">
+      <c r="I70" s="146"/>
+      <c r="J70" s="161"/>
+      <c r="K70" s="164">
         <f>ROUND(SUM(K66:K66),2)</f>
         <v>0</v>
       </c>
-      <c r="L70" s="148"/>
-      <c r="M70" s="168"/>
-      <c r="N70" s="149"/>
-      <c r="O70" s="150"/>
-      <c r="P70" s="171"/>
-      <c r="Q70" s="140"/>
-      <c r="R70" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S70" s="142"/>
-      <c r="T70" s="142"/>
-      <c r="U70" s="143" t="s">
+      <c r="L70" s="147"/>
+      <c r="M70" s="167"/>
+      <c r="N70" s="148"/>
+      <c r="O70" s="149"/>
+      <c r="P70" s="170"/>
+      <c r="Q70" s="139"/>
+      <c r="R70" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S70" s="141"/>
+      <c r="T70" s="141"/>
+      <c r="U70" s="142" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="71" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A71" s="151" t="s">
+      <c r="A71" s="150" t="s">
         <v>87</v>
       </c>
-      <c r="B71" s="152"/>
-      <c r="C71" s="153"/>
-      <c r="D71" s="154"/>
-      <c r="E71" s="154" t="s">
+      <c r="B71" s="151"/>
+      <c r="C71" s="152"/>
+      <c r="D71" s="153"/>
+      <c r="E71" s="153" t="s">
         <v>63</v>
       </c>
-      <c r="F71" s="154">
+      <c r="F71" s="153">
         <v>1</v>
       </c>
-      <c r="G71" s="160">
+      <c r="G71" s="159">
         <f>ROUND(H70,2)</f>
         <v>0</v>
       </c>
-      <c r="H71" s="160">
+      <c r="H71" s="159">
         <f>ROUND(F71*G71,0)</f>
         <v>0</v>
       </c>
-      <c r="I71" s="155"/>
-      <c r="J71" s="163"/>
-      <c r="K71" s="166">
+      <c r="I71" s="154"/>
+      <c r="J71" s="162"/>
+      <c r="K71" s="165">
         <f>ROUND(K70*F71,2)</f>
         <v>0</v>
       </c>
-      <c r="L71" s="156"/>
-      <c r="M71" s="169"/>
-      <c r="N71" s="157"/>
-      <c r="O71" s="158"/>
-      <c r="P71" s="172"/>
-      <c r="Q71" s="140"/>
-      <c r="R71" s="141" t="s">
-        <v>8</v>
-      </c>
-      <c r="S71" s="142"/>
-      <c r="T71" s="142"/>
-      <c r="U71" s="143" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="72" spans="1:21" s="128" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="L71" s="155"/>
+      <c r="M71" s="168"/>
+      <c r="N71" s="156"/>
+      <c r="O71" s="157"/>
+      <c r="P71" s="171"/>
+      <c r="Q71" s="139"/>
+      <c r="R71" s="140" t="s">
+        <v>8</v>
+      </c>
+      <c r="S71" s="141"/>
+      <c r="T71" s="141"/>
+      <c r="U71" s="142" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="72" spans="1:21" s="127" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A72" s="103"/>
-      <c r="B72" s="126" t="s">
-        <v>8</v>
-      </c>
-      <c r="C72" s="126" t="s">
-        <v>8</v>
-      </c>
-      <c r="D72" s="126" t="s">
+      <c r="B72" s="125" t="s">
+        <v>8</v>
+      </c>
+      <c r="C72" s="125" t="s">
+        <v>8</v>
+      </c>
+      <c r="D72" s="125" t="s">
         <v>8</v>
       </c>
       <c r="Q72" s="5"/>
       <c r="R72" s="5"/>
-      <c r="U72" s="126" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="73" spans="1:21" s="128" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="U72" s="125" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="73" spans="1:21" s="127" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A73" s="103"/>
-      <c r="B73" s="126" t="s">
-        <v>8</v>
-      </c>
-      <c r="C73" s="126" t="s">
-        <v>8</v>
-      </c>
-      <c r="D73" s="126" t="s">
+      <c r="B73" s="125" t="s">
+        <v>8</v>
+      </c>
+      <c r="C73" s="125" t="s">
+        <v>8</v>
+      </c>
+      <c r="D73" s="125" t="s">
         <v>8</v>
       </c>
       <c r="Q73" s="5"/>
       <c r="R73" s="5"/>
-      <c r="U73" s="126" t="s">
+      <c r="U73" s="125" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="74" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A74" s="173" t="str" cm="1">
-        <f t="array" aca="1" ref="A74" ca="1">CONCATENATE("报价人：", INDIRECT("项目信息!$B$8"))</f>
+      <c r="B74" s="172" t="str" cm="1">
+        <f t="array" aca="1" ref="B74" ca="1">CONCATENATE("报价人：", INDIRECT("项目信息!$B$8"))</f>
         <v>报价人：李四</v>
       </c>
-      <c r="B74" s="105"/>
-      <c r="C74" s="128"/>
-      <c r="D74" s="128"/>
-      <c r="E74" s="128"/>
-      <c r="F74" s="128"/>
-      <c r="G74" s="128"/>
-      <c r="H74" s="159" cm="1">
+      <c r="C74" s="127"/>
+      <c r="D74" s="127"/>
+      <c r="E74" s="127"/>
+      <c r="F74" s="127"/>
+      <c r="G74" s="127"/>
+      <c r="H74" s="158" cm="1">
         <f t="array" aca="1" ref="H74" ca="1">INDIRECT("项目信息!$B$9")</f>
         <v>0</v>
       </c>
       <c r="Q74" s="5"/>
       <c r="R74" s="5"/>
-      <c r="U74" s="135" t="s">
+      <c r="U74" s="134" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="75" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A75" s="159"/>
+      <c r="A75" s="158"/>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -5946,6 +5930,9 @@
       <formula1>"照明配电箱,动力配电箱,控制配电箱,电表箱,其它箱,动力柜,低压固定柜,低压抽屉柜,高压柜"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="A5:G5" location="项目信息!A29" display="项目信息!A29" xr:uid="{CE75005B-E606-4B3C-8176-67050F817366}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <customProperties>
     <customPr name="SCMID" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: add core modules for quotation check, cabinet pipeline, material stats, labor list, and finished handover
</commit_message>
<xml_diff>
--- a/Resources/CabinetTemplate.xlsx
+++ b/Resources/CabinetTemplate.xlsx
@@ -5,22 +5,30 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Ace\ExcelAddInCTtools\bin\Debug\net48\Resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\BaiduNetdiskWorkspace\BaseData\报价设置\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{609ADBB7-9E68-4855-B2B1-13A60C7D0A78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF595218-09A8-47DC-8D60-B0B8B8D9BA81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="15" windowWidth="19440" windowHeight="15000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="项目信息" sheetId="1" r:id="rId1"/>
-    <sheet name="分类1" sheetId="4" r:id="rId2"/>
+    <sheet name="领料清单" sheetId="5" r:id="rId1"/>
+    <sheet name="项目信息" sheetId="1" r:id="rId2"/>
+    <sheet name="分类1" sheetId="4" r:id="rId3"/>
+    <sheet name="采购清单" sheetId="6" r:id="rId4"/>
+    <sheet name="人工清单" sheetId="7" r:id="rId5"/>
+    <sheet name="成品交接单" sheetId="8" r:id="rId6"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId7"/>
+  </externalReferences>
   <definedNames>
     <definedName name="Cab_Det_1">分类1!$A$44</definedName>
     <definedName name="Cab_Subsum_1">分类1!$A$66</definedName>
     <definedName name="Cab_Sum_1">分类1!$A$7</definedName>
     <definedName name="Cab_Tolsum_1">分类1!$A$71</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">领料清单!$A$1:$L$15</definedName>
   </definedNames>
   <calcPr calcId="191029" concurrentCalc="0"/>
   <extLst>
@@ -62,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="158">
   <si>
     <t>序号</t>
     <phoneticPr fontId="6" type="noConversion"/>
@@ -479,12 +487,407 @@
     <t>台</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>成套设备装配领料单</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>工程名称 ：</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> [项目名称]</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">              </t>
+    </r>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>队组名称 ：</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ***  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">              </t>
+    </r>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>制表日期：</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>名称</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>型    号</t>
+  </si>
+  <si>
+    <t>单位</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>数量</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>生产厂家</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>领料人</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>备注</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>签字</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>[元器件名称]</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>[元器件型号]</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>[单位]</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>[数量]</t>
+  </si>
+  <si>
+    <t>[库存标记]</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>合计</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>编制人：</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">         编制复核人：          发货人</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>：</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">           发货复核人：           装配队组负责人</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>：</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">           </t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>[公司名称]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>名称</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>型号规格</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>单数</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>要求到货时间</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>合同到货时间</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>实际到货时间</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="24"/>
+        <rFont val="Microsoft YaHei UI"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>采  购</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="24"/>
+        <rFont val="楷体_GB2312"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> 清 单</t>
+    </r>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>[公司名称]</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>项目名称：[项目名称]</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>[元器件名称]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[型号]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[单位]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[数量]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[品牌]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>附件1：</t>
+  </si>
+  <si>
+    <t>人 工 清 单</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>队组：金旭彬/陈谦胜</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>型    号</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>单价（元）</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>金额（元）</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>配电箱</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>合计</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>台</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">   审核:                                 编制:                      日期:     年  月  日</t>
+  </si>
+  <si>
+    <t>成品交接单</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>单位名称：扬建集团机电分公司</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>队组：                调试人：              产成品入库：               日期：      年  月  日</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>项目名称：[[项目名称]]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[箱柜序号]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[箱柜名称]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[柜号]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[人工费]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>电流</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>防护等级</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>箱柜型号</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[箱柜型号]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[首行电流]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[分类名称]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="24"/>
+        <rFont val="Calibri"/>
+        <family val="3"/>
+      </rPr>
+      <t>[</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="24"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>公司名称</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="24"/>
+        <rFont val="Calibri"/>
+        <family val="3"/>
+      </rPr>
+      <t>]</t>
+    </r>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="8">
+  <numFmts count="11">
     <numFmt numFmtId="5" formatCode="&quot;¥&quot;#,##0;&quot;¥&quot;\-#,##0"/>
     <numFmt numFmtId="176" formatCode="0.00_ ;[Red]\-0.00\ "/>
     <numFmt numFmtId="177" formatCode="0.00_);[Red]\-0.00_)"/>
@@ -493,8 +896,11 @@
     <numFmt numFmtId="180" formatCode="&quot;备注:&quot;@"/>
     <numFmt numFmtId="181" formatCode="&quot;图号:&quot;@"/>
     <numFmt numFmtId="182" formatCode="0.00_);[Red]\(0.00\)"/>
+    <numFmt numFmtId="183" formatCode="m&quot;月&quot;d&quot;日&quot;;@"/>
+    <numFmt numFmtId="184" formatCode="0.0%"/>
+    <numFmt numFmtId="185" formatCode="0.00_ "/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="47">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -682,8 +1088,175 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="22"/>
+      <name val="楷体_GB2312"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <name val="楷体_GB2312"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="6"/>
+      <name val="楷体_GB2312"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <name val="Microsoft YaHei UI"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="22"/>
+      <name val="Microsoft YaHei UI"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <name val=""/>
+      <family val="1"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <name val="Calibri"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -768,8 +1341,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF6495ED"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="32">
+  <borders count="48">
     <border>
       <left/>
       <right/>
@@ -1162,16 +1741,242 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="217">
+  <cellXfs count="306">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1687,6 +2492,379 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="183" fontId="28" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="183" fontId="29" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="183" fontId="24" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="183" fontId="27" fillId="2" borderId="39" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="30" fillId="0" borderId="41" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="30" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="30" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="29" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="29" fillId="0" borderId="42" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="43" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="44" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="44" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="45" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="46" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="3" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="184" fontId="21" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="182" fontId="33" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="3" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="3" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="34" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="34" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="182" fontId="35" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="185" fontId="36" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="182" fontId="36" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="182" fontId="37" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="38" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="38" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="15" borderId="47" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="185" fontId="32" fillId="15" borderId="47" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="182" fontId="32" fillId="15" borderId="47" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="3" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="3" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="2" xfId="3" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="185" fontId="32" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="185" fontId="32" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="182" fontId="32" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="185" fontId="32" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="185" fontId="32" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="47" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="185" fontId="32" fillId="0" borderId="47" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="47" xfId="4" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="47" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="2" xfId="4" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="2" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="185" fontId="32" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="2" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="185" fontId="32" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="2" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="32" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="1" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="27" fillId="2" borderId="36" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="183" fontId="27" fillId="2" borderId="40" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="4" fillId="2" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="183" fontId="4" fillId="2" borderId="37" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="183" fontId="4" fillId="2" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="183" fontId="4" fillId="2" borderId="38" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="183" fontId="27" fillId="2" borderId="33" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="183" fontId="27" fillId="2" borderId="38" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="183" fontId="27" fillId="2" borderId="34" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="183" fontId="27" fillId="2" borderId="35" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1709,12 +2887,6 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
@@ -1752,86 +2924,16 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="5">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="常规 13" xfId="2" xr:uid="{99EDEE11-C2A1-4656-99EA-70988F2DB684}"/>
+    <cellStyle name="常规 2" xfId="3" xr:uid="{A622CDB6-4B9F-4954-897C-026C24A8ACB6}"/>
     <cellStyle name="超链接" xfId="1" builtinId="8"/>
+    <cellStyle name="超链接 2" xfId="4" xr:uid="{827C9D1E-13E0-4A75-A494-1B25858EF09F}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1954,6 +3056,41 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="领料清单"/>
+      <sheetName val="报价明细"/>
+      <sheetName val="报价汇总"/>
+      <sheetName val="人工清单"/>
+      <sheetName val="成品交接单"/>
+      <sheetName val="采购"/>
+      <sheetName val="二次图对应明细"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1">
+        <row r="4">
+          <cell r="A4" t="str">
+            <v>项目名称：GZ460</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2242,9 +3379,303 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D2842AD-2BE2-443E-91B2-38E6A2ECE42B}">
+  <sheetPr codeName="Sheet4"/>
+  <dimension ref="A1:AB17"/>
+  <sheetFormatPr defaultRowHeight="13.5"/>
+  <cols>
+    <col min="1" max="1" width="4.625" style="173" customWidth="1"/>
+    <col min="2" max="2" width="11.25" style="173" customWidth="1"/>
+    <col min="3" max="3" width="31.375" style="175" customWidth="1"/>
+    <col min="4" max="4" width="4.625" style="173" customWidth="1"/>
+    <col min="5" max="5" width="5.125" style="173" customWidth="1"/>
+    <col min="6" max="6" width="7.625" style="173" customWidth="1"/>
+    <col min="7" max="7" width="4.25" style="173" customWidth="1"/>
+    <col min="8" max="8" width="4.875" style="173" customWidth="1"/>
+    <col min="9" max="9" width="4.375" style="173" customWidth="1"/>
+    <col min="10" max="10" width="5.125" style="173" customWidth="1"/>
+    <col min="11" max="11" width="6.125" style="173" customWidth="1"/>
+    <col min="12" max="12" width="6.875" style="173" customWidth="1"/>
+    <col min="13" max="20" width="6.625" style="173" customWidth="1"/>
+    <col min="21" max="16384" width="9" style="173"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:28" ht="20.25">
+      <c r="A1" s="252" t="s">
+        <v>118</v>
+      </c>
+      <c r="B1" s="252"/>
+      <c r="C1" s="252"/>
+      <c r="D1" s="252"/>
+      <c r="E1" s="252"/>
+      <c r="F1" s="252"/>
+      <c r="G1" s="252"/>
+      <c r="H1" s="252"/>
+      <c r="I1" s="252"/>
+      <c r="J1" s="252"/>
+      <c r="K1" s="252"/>
+    </row>
+    <row r="2" spans="1:28" ht="20.25">
+      <c r="A2" s="252" t="s">
+        <v>98</v>
+      </c>
+      <c r="B2" s="252"/>
+      <c r="C2" s="252"/>
+      <c r="D2" s="252"/>
+      <c r="E2" s="252"/>
+      <c r="F2" s="252"/>
+      <c r="G2" s="252"/>
+      <c r="H2" s="252"/>
+      <c r="I2" s="252"/>
+      <c r="J2" s="252"/>
+      <c r="K2" s="252"/>
+    </row>
+    <row r="3" spans="1:28" ht="29.25" customHeight="1">
+      <c r="A3" s="174" t="s">
+        <v>99</v>
+      </c>
+      <c r="F3" s="174"/>
+      <c r="G3" s="174"/>
+      <c r="H3" s="174"/>
+      <c r="I3" s="174"/>
+      <c r="J3" s="174"/>
+      <c r="K3" s="174"/>
+    </row>
+    <row r="4" spans="1:28" ht="18" customHeight="1" thickBot="1">
+      <c r="A4" s="174" t="s">
+        <v>100</v>
+      </c>
+      <c r="F4" s="174" t="s">
+        <v>101</v>
+      </c>
+      <c r="G4" s="174"/>
+      <c r="H4" s="174"/>
+      <c r="I4" s="174"/>
+      <c r="J4" s="174"/>
+      <c r="K4" s="174"/>
+    </row>
+    <row r="5" spans="1:28" s="178" customFormat="1" ht="11.25" customHeight="1" thickBot="1">
+      <c r="A5" s="253" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="255" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5" s="255" t="s">
+        <v>103</v>
+      </c>
+      <c r="D5" s="255" t="s">
+        <v>104</v>
+      </c>
+      <c r="E5" s="255" t="s">
+        <v>105</v>
+      </c>
+      <c r="F5" s="257" t="s">
+        <v>106</v>
+      </c>
+      <c r="G5" s="259" t="s">
+        <v>107</v>
+      </c>
+      <c r="H5" s="260"/>
+      <c r="I5" s="259" t="s">
+        <v>107</v>
+      </c>
+      <c r="J5" s="260"/>
+      <c r="K5" s="250" t="s">
+        <v>108</v>
+      </c>
+      <c r="L5" s="176"/>
+      <c r="M5" s="176"/>
+      <c r="N5" s="176"/>
+      <c r="O5" s="176"/>
+      <c r="P5" s="176"/>
+      <c r="Q5" s="176"/>
+      <c r="R5" s="176"/>
+      <c r="S5" s="176"/>
+      <c r="T5" s="176"/>
+      <c r="U5" s="176"/>
+      <c r="V5" s="176"/>
+      <c r="W5" s="177"/>
+      <c r="X5" s="177"/>
+      <c r="Y5" s="177"/>
+      <c r="Z5" s="177"/>
+      <c r="AA5" s="177"/>
+      <c r="AB5" s="177"/>
+    </row>
+    <row r="6" spans="1:28" s="178" customFormat="1" ht="11.25" customHeight="1">
+      <c r="A6" s="254"/>
+      <c r="B6" s="256"/>
+      <c r="C6" s="256"/>
+      <c r="D6" s="256"/>
+      <c r="E6" s="256"/>
+      <c r="F6" s="258"/>
+      <c r="G6" s="179" t="s">
+        <v>105</v>
+      </c>
+      <c r="H6" s="179" t="s">
+        <v>109</v>
+      </c>
+      <c r="I6" s="179" t="s">
+        <v>105</v>
+      </c>
+      <c r="J6" s="179" t="s">
+        <v>109</v>
+      </c>
+      <c r="K6" s="251"/>
+      <c r="L6" s="176"/>
+      <c r="M6" s="176"/>
+      <c r="N6" s="176"/>
+      <c r="O6" s="176"/>
+      <c r="P6" s="176"/>
+      <c r="Q6" s="176"/>
+      <c r="R6" s="176"/>
+      <c r="S6" s="176"/>
+      <c r="T6" s="176"/>
+      <c r="U6" s="176"/>
+      <c r="V6" s="176"/>
+      <c r="W6" s="177"/>
+      <c r="X6" s="177"/>
+      <c r="Y6" s="177"/>
+      <c r="Z6" s="177"/>
+      <c r="AA6" s="177"/>
+      <c r="AB6" s="177"/>
+    </row>
+    <row r="7" spans="1:28" s="185" customFormat="1" ht="18.75" customHeight="1">
+      <c r="A7" s="180"/>
+      <c r="B7" s="181" t="s">
+        <v>110</v>
+      </c>
+      <c r="C7" s="181" t="s">
+        <v>111</v>
+      </c>
+      <c r="D7" s="181" t="s">
+        <v>112</v>
+      </c>
+      <c r="E7" s="181" t="s">
+        <v>113</v>
+      </c>
+      <c r="F7" s="181"/>
+      <c r="G7" s="182"/>
+      <c r="H7" s="182"/>
+      <c r="I7" s="183"/>
+      <c r="J7" s="183"/>
+      <c r="K7" s="184" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28" s="185" customFormat="1" ht="18" customHeight="1">
+      <c r="A8" s="180"/>
+      <c r="B8" s="181"/>
+      <c r="C8" s="181"/>
+      <c r="D8" s="181"/>
+      <c r="E8" s="181"/>
+      <c r="F8" s="181"/>
+      <c r="G8" s="182"/>
+      <c r="H8" s="182"/>
+      <c r="I8" s="183"/>
+      <c r="J8" s="183"/>
+      <c r="K8" s="184"/>
+    </row>
+    <row r="9" spans="1:28" s="185" customFormat="1" ht="18" customHeight="1">
+      <c r="A9" s="180"/>
+      <c r="B9" s="181"/>
+      <c r="C9" s="181"/>
+      <c r="D9" s="181"/>
+      <c r="E9" s="181"/>
+      <c r="F9" s="181"/>
+      <c r="G9" s="182"/>
+      <c r="H9" s="182"/>
+      <c r="I9" s="183"/>
+      <c r="J9" s="183"/>
+      <c r="K9" s="184"/>
+    </row>
+    <row r="10" spans="1:28" s="185" customFormat="1" ht="18" customHeight="1">
+      <c r="A10" s="180"/>
+      <c r="B10" s="181"/>
+      <c r="C10" s="181"/>
+      <c r="D10" s="181"/>
+      <c r="E10" s="181"/>
+      <c r="F10" s="181"/>
+      <c r="G10" s="182"/>
+      <c r="H10" s="182"/>
+      <c r="I10" s="183"/>
+      <c r="J10" s="183"/>
+      <c r="K10" s="184"/>
+    </row>
+    <row r="11" spans="1:28" ht="18" customHeight="1" thickBot="1">
+      <c r="A11" s="186"/>
+      <c r="B11" s="187" t="s">
+        <v>115</v>
+      </c>
+      <c r="C11" s="188"/>
+      <c r="D11" s="187"/>
+      <c r="E11" s="187"/>
+      <c r="F11" s="187"/>
+      <c r="G11" s="189"/>
+      <c r="H11" s="189"/>
+      <c r="I11" s="189"/>
+      <c r="J11" s="189"/>
+      <c r="K11" s="190"/>
+    </row>
+    <row r="12" spans="1:28" ht="18" customHeight="1"/>
+    <row r="13" spans="1:28" s="193" customFormat="1" ht="18" customHeight="1">
+      <c r="A13" s="174" t="s">
+        <v>116</v>
+      </c>
+      <c r="B13" s="191"/>
+      <c r="C13" s="192"/>
+      <c r="D13" s="173"/>
+      <c r="E13" s="173"/>
+      <c r="F13" s="173"/>
+      <c r="G13" s="173"/>
+      <c r="H13" s="173"/>
+      <c r="I13" s="173"/>
+      <c r="J13" s="173"/>
+      <c r="K13" s="173"/>
+    </row>
+    <row r="14" spans="1:28" ht="18" customHeight="1">
+      <c r="E14" s="194"/>
+      <c r="F14" s="194"/>
+      <c r="G14" s="194"/>
+      <c r="H14" s="194"/>
+      <c r="I14" s="194"/>
+      <c r="J14" s="194"/>
+      <c r="K14" s="194"/>
+    </row>
+    <row r="15" spans="1:28">
+      <c r="A15" s="173" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28" ht="20.100000000000001" customHeight="1"/>
+    <row r="17" ht="20.100000000000001" customHeight="1"/>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="I5:J5"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="171" orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddFooter>&amp;C第&amp;P页&amp;R共&amp;N页</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H59"/>
-  <sheetFormatPr defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultRowHeight="18" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
@@ -2255,27 +3686,27 @@
     <col min="7" max="8" width="13.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="195" t="str">
+    <row r="1" spans="1:8" ht="18" customHeight="1">
+      <c r="A1" s="264" t="str">
         <f>T(B22)</f>
         <v>扬州华科</v>
       </c>
-      <c r="B1" s="195"/>
-      <c r="C1" s="195"/>
-      <c r="D1" s="195"/>
+      <c r="B1" s="264"/>
+      <c r="C1" s="264"/>
+      <c r="D1" s="264"/>
       <c r="H1" s="1"/>
     </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="196" t="str">
+    <row r="2" spans="1:8" ht="18" customHeight="1">
+      <c r="A2" s="265" t="str">
         <f>T(B23)</f>
         <v/>
       </c>
-      <c r="B2" s="196"/>
-      <c r="C2" s="196"/>
-      <c r="D2" s="196"/>
+      <c r="B2" s="265"/>
+      <c r="C2" s="265"/>
+      <c r="D2" s="265"/>
       <c r="H2" s="1"/>
     </row>
-    <row r="3" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:8" ht="18" customHeight="1">
       <c r="A3" s="2"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -2285,25 +3716,25 @@
       <c r="G3" s="4"/>
       <c r="H3" s="5"/>
     </row>
-    <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="197" t="s">
+    <row r="4" spans="1:8" ht="18" customHeight="1">
+      <c r="A4" s="266" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="197"/>
-      <c r="C4" s="197"/>
-      <c r="D4" s="197"/>
-      <c r="E4" s="197"/>
-      <c r="F4" s="197"/>
+      <c r="B4" s="266"/>
+      <c r="C4" s="266"/>
+      <c r="D4" s="266"/>
+      <c r="E4" s="266"/>
+      <c r="F4" s="266"/>
       <c r="G4" s="4"/>
       <c r="H4" s="5"/>
     </row>
-    <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:8" ht="18" customHeight="1">
       <c r="A5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="198"/>
-      <c r="C5" s="199"/>
-      <c r="D5" s="200"/>
+      <c r="B5" s="267"/>
+      <c r="C5" s="268"/>
+      <c r="D5" s="269"/>
       <c r="E5" s="6" t="s">
         <v>7</v>
       </c>
@@ -2313,13 +3744,13 @@
       <c r="G5" s="4"/>
       <c r="H5" s="5"/>
     </row>
-    <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:8" ht="18" customHeight="1">
       <c r="A6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="180"/>
-      <c r="C6" s="194"/>
-      <c r="D6" s="181"/>
+      <c r="B6" s="261"/>
+      <c r="C6" s="262"/>
+      <c r="D6" s="263"/>
       <c r="E6" s="6" t="s">
         <v>10</v>
       </c>
@@ -2327,263 +3758,263 @@
       <c r="G6" s="4"/>
       <c r="H6" s="5"/>
     </row>
-    <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:8" ht="18" customHeight="1">
       <c r="A7" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="198"/>
-      <c r="C7" s="199"/>
-      <c r="D7" s="200"/>
+      <c r="B7" s="267"/>
+      <c r="C7" s="268"/>
+      <c r="D7" s="269"/>
       <c r="E7" s="9"/>
       <c r="F7" s="10"/>
       <c r="G7" s="4"/>
       <c r="H7" s="5"/>
     </row>
-    <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:8" ht="18" customHeight="1">
       <c r="A8" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="B8" s="180" t="s">
+      <c r="B8" s="261" t="s">
         <v>94</v>
       </c>
-      <c r="C8" s="194"/>
-      <c r="D8" s="181"/>
+      <c r="C8" s="262"/>
+      <c r="D8" s="263"/>
       <c r="E8" s="11"/>
       <c r="F8" s="12"/>
       <c r="G8" s="4"/>
       <c r="H8" s="5"/>
     </row>
-    <row r="9" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:8" ht="18" customHeight="1">
       <c r="A9" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="180"/>
-      <c r="C9" s="194"/>
-      <c r="D9" s="181"/>
+      <c r="B9" s="261"/>
+      <c r="C9" s="262"/>
+      <c r="D9" s="263"/>
       <c r="E9" s="11"/>
       <c r="F9" s="12"/>
       <c r="G9" s="4"/>
       <c r="H9" s="5"/>
     </row>
-    <row r="10" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:8" ht="18" customHeight="1">
       <c r="A10" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="180"/>
-      <c r="C10" s="194"/>
-      <c r="D10" s="181"/>
+      <c r="B10" s="261"/>
+      <c r="C10" s="262"/>
+      <c r="D10" s="263"/>
       <c r="E10" s="11"/>
       <c r="F10" s="12"/>
       <c r="G10" s="4"/>
       <c r="H10" s="5"/>
     </row>
-    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:8" ht="18" customHeight="1">
       <c r="A11" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="180"/>
-      <c r="C11" s="194"/>
-      <c r="D11" s="181"/>
+      <c r="B11" s="261"/>
+      <c r="C11" s="262"/>
+      <c r="D11" s="263"/>
       <c r="E11" s="11"/>
       <c r="F11" s="12"/>
       <c r="G11" s="4"/>
       <c r="H11" s="5"/>
     </row>
-    <row r="12" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:8" ht="18" customHeight="1">
       <c r="A12" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="180"/>
-      <c r="C12" s="194"/>
-      <c r="D12" s="181"/>
+      <c r="B12" s="261"/>
+      <c r="C12" s="262"/>
+      <c r="D12" s="263"/>
       <c r="E12" s="11"/>
       <c r="F12" s="12"/>
       <c r="G12" s="4"/>
       <c r="H12" s="5"/>
     </row>
-    <row r="13" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A13" s="201" t="s">
+    <row r="13" spans="1:8" ht="18" customHeight="1">
+      <c r="A13" s="270" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="202"/>
-      <c r="C13" s="202"/>
-      <c r="D13" s="203"/>
+      <c r="B13" s="271"/>
+      <c r="C13" s="271"/>
+      <c r="D13" s="272"/>
       <c r="E13" s="11"/>
       <c r="F13" s="12"/>
       <c r="G13" s="4"/>
       <c r="H13" s="5"/>
     </row>
-    <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:8" ht="18" customHeight="1">
       <c r="A14" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="180"/>
-      <c r="C14" s="194"/>
-      <c r="D14" s="181"/>
+      <c r="B14" s="261"/>
+      <c r="C14" s="262"/>
+      <c r="D14" s="263"/>
       <c r="E14" s="11"/>
       <c r="F14" s="12"/>
       <c r="G14" s="4"/>
       <c r="H14" s="5"/>
     </row>
-    <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:8" ht="18" customHeight="1">
       <c r="A15" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="180"/>
-      <c r="C15" s="194"/>
-      <c r="D15" s="181"/>
+      <c r="B15" s="261"/>
+      <c r="C15" s="262"/>
+      <c r="D15" s="263"/>
       <c r="E15" s="11"/>
       <c r="F15" s="12"/>
       <c r="G15" s="4"/>
       <c r="H15" s="5"/>
     </row>
-    <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:8" ht="18" customHeight="1">
       <c r="A16" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="180"/>
-      <c r="C16" s="194"/>
-      <c r="D16" s="181"/>
+      <c r="B16" s="261"/>
+      <c r="C16" s="262"/>
+      <c r="D16" s="263"/>
       <c r="E16" s="11"/>
       <c r="F16" s="12"/>
       <c r="G16" s="4"/>
       <c r="H16" s="5"/>
     </row>
-    <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:8" ht="18" customHeight="1">
       <c r="A17" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="180"/>
-      <c r="C17" s="194"/>
-      <c r="D17" s="181"/>
+      <c r="B17" s="261"/>
+      <c r="C17" s="262"/>
+      <c r="D17" s="263"/>
       <c r="E17" s="11"/>
       <c r="F17" s="12"/>
       <c r="G17" s="4"/>
       <c r="H17" s="5"/>
     </row>
-    <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:8" ht="18" customHeight="1">
       <c r="A18" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="180"/>
-      <c r="C18" s="194"/>
-      <c r="D18" s="181"/>
+      <c r="B18" s="261"/>
+      <c r="C18" s="262"/>
+      <c r="D18" s="263"/>
       <c r="E18" s="11"/>
       <c r="F18" s="12"/>
       <c r="G18" s="4"/>
       <c r="H18" s="5"/>
     </row>
-    <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:8" ht="18" customHeight="1">
       <c r="A19" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="180"/>
-      <c r="C19" s="194"/>
-      <c r="D19" s="181"/>
+      <c r="B19" s="261"/>
+      <c r="C19" s="262"/>
+      <c r="D19" s="263"/>
       <c r="E19" s="11"/>
       <c r="F19" s="12"/>
       <c r="G19" s="4"/>
       <c r="H19" s="5"/>
     </row>
-    <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:8" ht="18" customHeight="1">
       <c r="A20" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="180"/>
-      <c r="C20" s="194"/>
-      <c r="D20" s="181"/>
+      <c r="B20" s="261"/>
+      <c r="C20" s="262"/>
+      <c r="D20" s="263"/>
       <c r="E20" s="11"/>
       <c r="F20" s="12"/>
       <c r="G20" s="4"/>
       <c r="H20" s="5"/>
     </row>
-    <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A21" s="201" t="s">
+    <row r="21" spans="1:8" ht="18" customHeight="1">
+      <c r="A21" s="270" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="202"/>
-      <c r="C21" s="202"/>
-      <c r="D21" s="203"/>
+      <c r="B21" s="271"/>
+      <c r="C21" s="271"/>
+      <c r="D21" s="272"/>
       <c r="E21" s="11"/>
       <c r="F21" s="12"/>
       <c r="G21" s="4"/>
       <c r="H21" s="5"/>
     </row>
-    <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:8" ht="18" customHeight="1">
       <c r="A22" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B22" s="180" t="s">
+      <c r="B22" s="261" t="s">
         <v>95</v>
       </c>
-      <c r="C22" s="194"/>
-      <c r="D22" s="181"/>
+      <c r="C22" s="262"/>
+      <c r="D22" s="263"/>
       <c r="E22" s="11"/>
       <c r="F22" s="12"/>
       <c r="G22" s="4"/>
       <c r="H22" s="5"/>
     </row>
-    <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:8" ht="18" customHeight="1">
       <c r="A23" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="180"/>
-      <c r="C23" s="194"/>
-      <c r="D23" s="181"/>
+      <c r="B23" s="261"/>
+      <c r="C23" s="262"/>
+      <c r="D23" s="263"/>
       <c r="E23" s="11"/>
       <c r="F23" s="12"/>
       <c r="G23" s="4"/>
       <c r="H23" s="5"/>
     </row>
-    <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:8" ht="18" customHeight="1">
       <c r="A24" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B24" s="180"/>
-      <c r="C24" s="194"/>
-      <c r="D24" s="181"/>
+      <c r="B24" s="261"/>
+      <c r="C24" s="262"/>
+      <c r="D24" s="263"/>
       <c r="E24" s="11"/>
       <c r="F24" s="12"/>
       <c r="G24" s="4"/>
       <c r="H24" s="5"/>
     </row>
-    <row r="25" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:8" ht="18" customHeight="1">
       <c r="A25" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B25" s="180"/>
-      <c r="C25" s="194"/>
-      <c r="D25" s="181"/>
+      <c r="B25" s="261"/>
+      <c r="C25" s="262"/>
+      <c r="D25" s="263"/>
       <c r="E25" s="11"/>
       <c r="F25" s="12"/>
       <c r="G25" s="4"/>
       <c r="H25" s="5"/>
     </row>
-    <row r="26" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:8" ht="18" customHeight="1">
       <c r="A26" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B26" s="180"/>
-      <c r="C26" s="194"/>
-      <c r="D26" s="181"/>
+      <c r="B26" s="261"/>
+      <c r="C26" s="262"/>
+      <c r="D26" s="263"/>
       <c r="E26" s="11"/>
       <c r="F26" s="12"/>
       <c r="G26" s="4"/>
       <c r="H26" s="5"/>
     </row>
-    <row r="27" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A27" s="204" t="s">
+    <row r="27" spans="1:8" ht="18" customHeight="1">
+      <c r="A27" s="273" t="s">
         <v>28</v>
       </c>
-      <c r="B27" s="205"/>
-      <c r="C27" s="205"/>
-      <c r="D27" s="206"/>
+      <c r="B27" s="274"/>
+      <c r="C27" s="274"/>
+      <c r="D27" s="275"/>
       <c r="E27" s="13"/>
       <c r="F27" s="14"/>
       <c r="G27" s="4"/>
       <c r="H27" s="5"/>
     </row>
-    <row r="28" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:8" ht="18" customHeight="1">
       <c r="A28" s="15" t="s">
         <v>29</v>
       </c>
@@ -2609,7 +4040,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:8" ht="18" customHeight="1">
       <c r="A29" s="107">
         <f t="shared" ref="A29:A56" si="0">ROW()-ROW(A$28)</f>
         <v>1</v>
@@ -2643,7 +4074,7 @@
         <v>常规</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:8" ht="18" customHeight="1">
       <c r="A30" s="28">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -2656,7 +4087,7 @@
       <c r="G30" s="34"/>
       <c r="H30" s="27"/>
     </row>
-    <row r="31" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:8" ht="18" customHeight="1">
       <c r="A31" s="28">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -2669,7 +4100,7 @@
       <c r="G31" s="34"/>
       <c r="H31" s="27"/>
     </row>
-    <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:8" ht="18" customHeight="1">
       <c r="A32" s="28">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -2682,7 +4113,7 @@
       <c r="G32" s="34"/>
       <c r="H32" s="27"/>
     </row>
-    <row r="33" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:8" ht="18" customHeight="1">
       <c r="A33" s="28">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -2695,7 +4126,7 @@
       <c r="G33" s="34"/>
       <c r="H33" s="27"/>
     </row>
-    <row r="34" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:8" ht="18" customHeight="1">
       <c r="A34" s="28">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -2708,7 +4139,7 @@
       <c r="G34" s="34"/>
       <c r="H34" s="27"/>
     </row>
-    <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:8" ht="18" customHeight="1">
       <c r="A35" s="28">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -2721,7 +4152,7 @@
       <c r="G35" s="34"/>
       <c r="H35" s="27"/>
     </row>
-    <row r="36" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:8" ht="18" customHeight="1">
       <c r="A36" s="28">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -2734,7 +4165,7 @@
       <c r="G36" s="34"/>
       <c r="H36" s="27"/>
     </row>
-    <row r="37" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:8" ht="18" customHeight="1">
       <c r="A37" s="28">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -2747,7 +4178,7 @@
       <c r="G37" s="34"/>
       <c r="H37" s="27"/>
     </row>
-    <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:8" ht="18" customHeight="1">
       <c r="A38" s="28">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -2760,7 +4191,7 @@
       <c r="G38" s="34"/>
       <c r="H38" s="27"/>
     </row>
-    <row r="39" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:8" ht="18" customHeight="1">
       <c r="A39" s="28">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -2773,7 +4204,7 @@
       <c r="G39" s="34"/>
       <c r="H39" s="27"/>
     </row>
-    <row r="40" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:8" ht="18" customHeight="1">
       <c r="A40" s="28">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -2786,7 +4217,7 @@
       <c r="G40" s="34"/>
       <c r="H40" s="27"/>
     </row>
-    <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:8" ht="18" customHeight="1">
       <c r="A41" s="28">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -2799,7 +4230,7 @@
       <c r="G41" s="34"/>
       <c r="H41" s="27"/>
     </row>
-    <row r="42" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="42" spans="1:8" ht="18" customHeight="1">
       <c r="A42" s="28">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -2812,7 +4243,7 @@
       <c r="G42" s="34"/>
       <c r="H42" s="27"/>
     </row>
-    <row r="43" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:8" ht="18" customHeight="1">
       <c r="A43" s="28">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -2825,7 +4256,7 @@
       <c r="G43" s="34"/>
       <c r="H43" s="27"/>
     </row>
-    <row r="44" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="44" spans="1:8" ht="18" customHeight="1">
       <c r="A44" s="28">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -2838,7 +4269,7 @@
       <c r="G44" s="34"/>
       <c r="H44" s="27"/>
     </row>
-    <row r="45" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:8" ht="18" customHeight="1">
       <c r="A45" s="28">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -2851,7 +4282,7 @@
       <c r="G45" s="34"/>
       <c r="H45" s="27"/>
     </row>
-    <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="46" spans="1:8" ht="18" customHeight="1">
       <c r="A46" s="28">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -2864,7 +4295,7 @@
       <c r="G46" s="34"/>
       <c r="H46" s="27"/>
     </row>
-    <row r="47" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="47" spans="1:8" ht="18" customHeight="1">
       <c r="A47" s="28">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -2877,7 +4308,7 @@
       <c r="G47" s="34"/>
       <c r="H47" s="27"/>
     </row>
-    <row r="48" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="48" spans="1:8" ht="18" customHeight="1">
       <c r="A48" s="28">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -2890,7 +4321,7 @@
       <c r="G48" s="34"/>
       <c r="H48" s="27"/>
     </row>
-    <row r="49" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="49" spans="1:8" ht="18" customHeight="1">
       <c r="A49" s="28">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -2903,7 +4334,7 @@
       <c r="G49" s="34"/>
       <c r="H49" s="27"/>
     </row>
-    <row r="50" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="50" spans="1:8" ht="18" customHeight="1">
       <c r="A50" s="28">
         <f t="shared" si="0"/>
         <v>22</v>
@@ -2916,7 +4347,7 @@
       <c r="G50" s="34"/>
       <c r="H50" s="27"/>
     </row>
-    <row r="51" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="51" spans="1:8" ht="18" customHeight="1">
       <c r="A51" s="28">
         <f t="shared" si="0"/>
         <v>23</v>
@@ -2929,7 +4360,7 @@
       <c r="G51" s="34"/>
       <c r="H51" s="27"/>
     </row>
-    <row r="52" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="52" spans="1:8" ht="18" customHeight="1">
       <c r="A52" s="28">
         <f t="shared" si="0"/>
         <v>24</v>
@@ -2942,7 +4373,7 @@
       <c r="G52" s="34"/>
       <c r="H52" s="27"/>
     </row>
-    <row r="53" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="53" spans="1:8" ht="18" customHeight="1">
       <c r="A53" s="28">
         <f t="shared" si="0"/>
         <v>25</v>
@@ -2975,7 +4406,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="54" spans="1:8" ht="18" customHeight="1">
       <c r="A54" s="28">
         <f t="shared" si="0"/>
         <v>26</v>
@@ -2992,7 +4423,7 @@
       <c r="G54" s="45"/>
       <c r="H54" s="42"/>
     </row>
-    <row r="55" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="55" spans="1:8" ht="18" customHeight="1">
       <c r="A55" s="46">
         <f t="shared" si="0"/>
         <v>27</v>
@@ -3010,7 +4441,7 @@
       <c r="G55" s="52"/>
       <c r="H55" s="53"/>
     </row>
-    <row r="56" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="56" spans="1:8" ht="18" customHeight="1">
       <c r="A56" s="46">
         <f t="shared" si="0"/>
         <v>28</v>
@@ -3018,39 +4449,39 @@
       <c r="B56" s="47" t="s">
         <v>40</v>
       </c>
-      <c r="C56" s="207" t="str">
+      <c r="C56" s="276" t="str">
         <f ca="1">TEXT(SUBSTITUTE(IF(D55="","",IF(MOD(D55,1)=0,TEXT(INT(D55),"[DBNum2][$-804]G/通用格式元整"),(TEXT(INT(D55),"[DBNum2][$-804]G/通用格式元")&amp;TEXT((INT(D55*10)-INT(D55)*10),"[DBNum2][$-804]G/通用格式角")&amp;TEXT((INT(D55*100)-INT(D55*10)*10),"[DBNum2][$-804]G/通用格式分")))),"零角","零"),)</f>
         <v>零元整</v>
       </c>
-      <c r="D56" s="208"/>
+      <c r="D56" s="277"/>
       <c r="E56" s="4"/>
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
       <c r="H56" s="5"/>
     </row>
-    <row r="57" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A57" s="209" t="s">
+    <row r="57" spans="1:8" ht="18" customHeight="1">
+      <c r="A57" s="278" t="s">
         <v>41</v>
       </c>
-      <c r="B57" s="211"/>
-      <c r="C57" s="212"/>
-      <c r="D57" s="213"/>
+      <c r="B57" s="280"/>
+      <c r="C57" s="281"/>
+      <c r="D57" s="282"/>
       <c r="E57" s="4"/>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
       <c r="H57" s="5"/>
     </row>
-    <row r="58" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A58" s="210"/>
-      <c r="B58" s="214"/>
-      <c r="C58" s="215"/>
-      <c r="D58" s="216"/>
+    <row r="58" spans="1:8" ht="18" customHeight="1">
+      <c r="A58" s="279"/>
+      <c r="B58" s="283"/>
+      <c r="C58" s="284"/>
+      <c r="D58" s="285"/>
       <c r="E58" s="4"/>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
       <c r="H58" s="5"/>
     </row>
-    <row r="59" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="59" spans="1:8" ht="18" customHeight="1">
       <c r="A59" s="54"/>
       <c r="B59" s="55"/>
       <c r="C59" s="55"/>
@@ -3110,10 +4541,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64F42C16-0E02-45B5-8A6E-93E7DC082CF9}">
   <dimension ref="A1:U75"/>
-  <sheetFormatPr defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultRowHeight="18" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="13.625" customWidth="1"/>
@@ -3133,68 +4564,68 @@
     <col min="25" max="25" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:17" ht="18" customHeight="1">
       <c r="A1" s="57"/>
       <c r="F1" s="58"/>
       <c r="I1" s="58"/>
     </row>
-    <row r="2" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="174" t="str">
+    <row r="2" spans="1:17" ht="18" customHeight="1">
+      <c r="A2" s="287" t="str">
         <f ca="1">T(INDIRECT("项目信息!B22"))</f>
         <v>扬州华科</v>
       </c>
-      <c r="B2" s="174"/>
-      <c r="C2" s="174"/>
-      <c r="D2" s="174"/>
-      <c r="E2" s="174"/>
-      <c r="F2" s="174"/>
-      <c r="G2" s="174"/>
-      <c r="H2" s="174"/>
-      <c r="I2" s="174"/>
-    </row>
-    <row r="3" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="174" t="str">
+      <c r="B2" s="287"/>
+      <c r="C2" s="287"/>
+      <c r="D2" s="287"/>
+      <c r="E2" s="287"/>
+      <c r="F2" s="287"/>
+      <c r="G2" s="287"/>
+      <c r="H2" s="287"/>
+      <c r="I2" s="287"/>
+    </row>
+    <row r="3" spans="1:17" ht="18" customHeight="1">
+      <c r="A3" s="287" t="str">
         <f ca="1">T(INDIRECT("项目信息!B23"))</f>
         <v/>
       </c>
-      <c r="B3" s="174"/>
-      <c r="C3" s="174"/>
-      <c r="D3" s="174"/>
-      <c r="E3" s="174"/>
-      <c r="F3" s="174"/>
-      <c r="G3" s="174"/>
-      <c r="H3" s="174"/>
-      <c r="I3" s="174"/>
-    </row>
-    <row r="4" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="175" t="s">
+      <c r="B3" s="287"/>
+      <c r="C3" s="287"/>
+      <c r="D3" s="287"/>
+      <c r="E3" s="287"/>
+      <c r="F3" s="287"/>
+      <c r="G3" s="287"/>
+      <c r="H3" s="287"/>
+      <c r="I3" s="287"/>
+    </row>
+    <row r="4" spans="1:17" ht="18" customHeight="1">
+      <c r="A4" s="288" t="s">
         <v>42</v>
       </c>
-      <c r="B4" s="176"/>
-      <c r="C4" s="176"/>
-      <c r="D4" s="176"/>
-      <c r="E4" s="176"/>
-      <c r="F4" s="176"/>
-      <c r="G4" s="176"/>
-      <c r="H4" s="176"/>
-      <c r="I4" s="176"/>
-    </row>
-    <row r="5" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="177" t="str" cm="1">
+      <c r="B4" s="289"/>
+      <c r="C4" s="289"/>
+      <c r="D4" s="289"/>
+      <c r="E4" s="289"/>
+      <c r="F4" s="289"/>
+      <c r="G4" s="289"/>
+      <c r="H4" s="289"/>
+      <c r="I4" s="289"/>
+    </row>
+    <row r="5" spans="1:17" ht="18" customHeight="1">
+      <c r="A5" s="290" t="str" cm="1">
         <f t="array" aca="1" ref="A5" ca="1">CONCATENATE("项目名称:",INDIRECT("项目信息!$B$5"))</f>
         <v>项目名称:</v>
       </c>
-      <c r="B5" s="178"/>
-      <c r="C5" s="178"/>
-      <c r="D5" s="178"/>
-      <c r="E5" s="178"/>
-      <c r="F5" s="178"/>
-      <c r="G5" s="179"/>
-      <c r="H5" s="180" t="str">
+      <c r="B5" s="291"/>
+      <c r="C5" s="291"/>
+      <c r="D5" s="291"/>
+      <c r="E5" s="291"/>
+      <c r="F5" s="291"/>
+      <c r="G5" s="292"/>
+      <c r="H5" s="261" t="str">
         <f ca="1">CONCATENATE("报价序号:", INDIRECT("'项目信息'!B7"))</f>
         <v>报价序号:</v>
       </c>
-      <c r="I5" s="181"/>
+      <c r="I5" s="263"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
@@ -3204,7 +4635,7 @@
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
     </row>
-    <row r="6" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:17" ht="18" customHeight="1">
       <c r="A6" s="15" t="s">
         <v>0</v>
       </c>
@@ -3257,7 +4688,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:17" ht="18" customHeight="1">
       <c r="A7" s="46">
         <f>ROW()-ROW(A$6)</f>
         <v>1</v>
@@ -3285,7 +4716,7 @@
       <c r="P7" s="74"/>
       <c r="Q7" s="75"/>
     </row>
-    <row r="8" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:17" ht="18" customHeight="1">
       <c r="A8" s="46">
         <f t="shared" ref="A8:A35" si="0">ROW()-ROW(A$6)</f>
         <v>2</v>
@@ -3307,7 +4738,7 @@
       <c r="P8" s="74"/>
       <c r="Q8" s="75"/>
     </row>
-    <row r="9" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:17" ht="18" customHeight="1">
       <c r="A9" s="46">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -3329,7 +4760,7 @@
       <c r="P9" s="74"/>
       <c r="Q9" s="75"/>
     </row>
-    <row r="10" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:17" ht="18" customHeight="1">
       <c r="A10" s="46">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -3351,7 +4782,7 @@
       <c r="P10" s="74"/>
       <c r="Q10" s="75"/>
     </row>
-    <row r="11" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:17" ht="18" customHeight="1">
       <c r="A11" s="46">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -3373,7 +4804,7 @@
       <c r="P11" s="74"/>
       <c r="Q11" s="75"/>
     </row>
-    <row r="12" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:17" ht="18" customHeight="1">
       <c r="A12" s="46">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -3395,7 +4826,7 @@
       <c r="P12" s="74"/>
       <c r="Q12" s="75"/>
     </row>
-    <row r="13" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:17" ht="18" customHeight="1">
       <c r="A13" s="46">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -3417,7 +4848,7 @@
       <c r="P13" s="74"/>
       <c r="Q13" s="75"/>
     </row>
-    <row r="14" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:17" ht="18" customHeight="1">
       <c r="A14" s="46">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -3439,7 +4870,7 @@
       <c r="P14" s="74"/>
       <c r="Q14" s="75"/>
     </row>
-    <row r="15" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:17" ht="18" customHeight="1">
       <c r="A15" s="46">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -3461,7 +4892,7 @@
       <c r="P15" s="74"/>
       <c r="Q15" s="75"/>
     </row>
-    <row r="16" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:17" ht="18" customHeight="1">
       <c r="A16" s="46">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -3483,7 +4914,7 @@
       <c r="P16" s="74"/>
       <c r="Q16" s="75"/>
     </row>
-    <row r="17" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:17" ht="18" customHeight="1">
       <c r="A17" s="46">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -3505,7 +4936,7 @@
       <c r="P17" s="74"/>
       <c r="Q17" s="75"/>
     </row>
-    <row r="18" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:17" ht="18" customHeight="1">
       <c r="A18" s="46">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -3527,7 +4958,7 @@
       <c r="P18" s="74"/>
       <c r="Q18" s="75"/>
     </row>
-    <row r="19" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:17" ht="18" customHeight="1">
       <c r="A19" s="46">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -3549,7 +4980,7 @@
       <c r="P19" s="74"/>
       <c r="Q19" s="75"/>
     </row>
-    <row r="20" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:17" ht="18" customHeight="1">
       <c r="A20" s="46">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -3571,7 +5002,7 @@
       <c r="P20" s="74"/>
       <c r="Q20" s="75"/>
     </row>
-    <row r="21" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:17" ht="18" customHeight="1">
       <c r="A21" s="46">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -3593,7 +5024,7 @@
       <c r="P21" s="74"/>
       <c r="Q21" s="75"/>
     </row>
-    <row r="22" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:17" ht="18" customHeight="1">
       <c r="A22" s="46">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -3615,7 +5046,7 @@
       <c r="P22" s="74"/>
       <c r="Q22" s="75"/>
     </row>
-    <row r="23" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:17" ht="18" customHeight="1">
       <c r="A23" s="46">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -3637,7 +5068,7 @@
       <c r="P23" s="74"/>
       <c r="Q23" s="75"/>
     </row>
-    <row r="24" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:17" ht="18" customHeight="1">
       <c r="A24" s="46">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -3659,7 +5090,7 @@
       <c r="P24" s="74"/>
       <c r="Q24" s="75"/>
     </row>
-    <row r="25" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:17" ht="18" customHeight="1">
       <c r="A25" s="46">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -3681,7 +5112,7 @@
       <c r="P25" s="74"/>
       <c r="Q25" s="75"/>
     </row>
-    <row r="26" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:17" ht="18" customHeight="1">
       <c r="A26" s="46">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -3703,7 +5134,7 @@
       <c r="P26" s="74"/>
       <c r="Q26" s="75"/>
     </row>
-    <row r="27" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:17" ht="18" customHeight="1">
       <c r="A27" s="46">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -3725,7 +5156,7 @@
       <c r="P27" s="74"/>
       <c r="Q27" s="75"/>
     </row>
-    <row r="28" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:17" ht="18" customHeight="1">
       <c r="A28" s="46">
         <f t="shared" si="0"/>
         <v>22</v>
@@ -3747,7 +5178,7 @@
       <c r="P28" s="74"/>
       <c r="Q28" s="75"/>
     </row>
-    <row r="29" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:17" ht="18" customHeight="1">
       <c r="A29" s="46">
         <f t="shared" si="0"/>
         <v>23</v>
@@ -3769,7 +5200,7 @@
       <c r="P29" s="74"/>
       <c r="Q29" s="75"/>
     </row>
-    <row r="30" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:17" ht="18" customHeight="1">
       <c r="A30" s="46">
         <f t="shared" si="0"/>
         <v>24</v>
@@ -3791,7 +5222,7 @@
       <c r="P30" s="74"/>
       <c r="Q30" s="75"/>
     </row>
-    <row r="31" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:17" ht="18" customHeight="1">
       <c r="A31" s="46">
         <f t="shared" si="0"/>
         <v>25</v>
@@ -3829,7 +5260,7 @@
       <c r="P31" s="74"/>
       <c r="Q31" s="75"/>
     </row>
-    <row r="32" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:17" ht="18" customHeight="1">
       <c r="A32" s="46">
         <f t="shared" si="0"/>
         <v>26</v>
@@ -3865,7 +5296,7 @@
       <c r="P32" s="74"/>
       <c r="Q32" s="90"/>
     </row>
-    <row r="33" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:21" ht="18" customHeight="1">
       <c r="A33" s="46">
         <f t="shared" si="0"/>
         <v>27</v>
@@ -3901,7 +5332,7 @@
       <c r="P33" s="74"/>
       <c r="Q33" s="90"/>
     </row>
-    <row r="34" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:21" ht="18" customHeight="1">
       <c r="A34" s="46">
         <f t="shared" si="0"/>
         <v>28</v>
@@ -3937,7 +5368,7 @@
       <c r="P34" s="74"/>
       <c r="Q34" s="90"/>
     </row>
-    <row r="35" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:21" ht="18" customHeight="1">
       <c r="A35" s="46">
         <f t="shared" si="0"/>
         <v>29</v>
@@ -3945,11 +5376,11 @@
       <c r="B35" s="92" t="s">
         <v>60</v>
       </c>
-      <c r="C35" s="182" t="str">
+      <c r="C35" s="293" t="str">
         <f ca="1">TEXT(SUBSTITUTE(IF(H35="","",IF(MOD(H35,1)=0,TEXT(INT(H35),"[DBNum2][$-804]G/通用格式元整"),(TEXT(INT(H35),"[DBNum2][$-804]G/通用格式元")&amp;TEXT((INT(H35*10)-INT(H35)*10),"[DBNum2][$-804]G/通用格式角")&amp;TEXT((INT(H35*100)-INT(H35*10)*10),"[DBNum2][$-804]G/通用格式分")))),"零角","零"),)</f>
         <v>零元整</v>
       </c>
-      <c r="D35" s="183"/>
+      <c r="D35" s="294"/>
       <c r="E35" s="93"/>
       <c r="F35" s="94" t="str">
         <f ca="1">IF(INDIRECT("'项目信息'!H29")="箱变", 1, "")</f>
@@ -3982,18 +5413,18 @@
       <c r="P35" s="100"/>
       <c r="Q35" s="101"/>
     </row>
-    <row r="36" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A36" s="184" t="s">
+    <row r="36" spans="1:21" ht="18" customHeight="1">
+      <c r="A36" s="295" t="s">
         <v>61</v>
       </c>
-      <c r="B36" s="186"/>
-      <c r="C36" s="187"/>
-      <c r="D36" s="187"/>
-      <c r="E36" s="187"/>
-      <c r="F36" s="187"/>
-      <c r="G36" s="188"/>
-      <c r="H36" s="188"/>
-      <c r="I36" s="189"/>
+      <c r="B36" s="297"/>
+      <c r="C36" s="298"/>
+      <c r="D36" s="298"/>
+      <c r="E36" s="298"/>
+      <c r="F36" s="298"/>
+      <c r="G36" s="299"/>
+      <c r="H36" s="299"/>
+      <c r="I36" s="300"/>
       <c r="J36" s="114"/>
       <c r="K36" s="114"/>
       <c r="L36" s="4"/>
@@ -4003,16 +5434,16 @@
       <c r="P36" s="4"/>
       <c r="Q36" s="4"/>
     </row>
-    <row r="37" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A37" s="185"/>
-      <c r="B37" s="190"/>
-      <c r="C37" s="190"/>
-      <c r="D37" s="190"/>
-      <c r="E37" s="190"/>
-      <c r="F37" s="190"/>
-      <c r="G37" s="191"/>
-      <c r="H37" s="191"/>
-      <c r="I37" s="192"/>
+    <row r="37" spans="1:21" ht="18" customHeight="1">
+      <c r="A37" s="296"/>
+      <c r="B37" s="301"/>
+      <c r="C37" s="301"/>
+      <c r="D37" s="301"/>
+      <c r="E37" s="301"/>
+      <c r="F37" s="301"/>
+      <c r="G37" s="302"/>
+      <c r="H37" s="302"/>
+      <c r="I37" s="303"/>
       <c r="J37" s="114"/>
       <c r="K37" s="114"/>
       <c r="L37" s="4"/>
@@ -4022,7 +5453,7 @@
       <c r="P37" s="4"/>
       <c r="Q37" s="4"/>
     </row>
-    <row r="38" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:21" ht="18" customHeight="1">
       <c r="A38" s="103"/>
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
@@ -4041,7 +5472,7 @@
       <c r="P38" s="4"/>
       <c r="Q38" s="4"/>
     </row>
-    <row r="39" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:21" ht="18" customHeight="1">
       <c r="A39" s="103"/>
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
@@ -4060,7 +5491,7 @@
       <c r="P39" s="4"/>
       <c r="Q39" s="4"/>
     </row>
-    <row r="40" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:21" ht="18" customHeight="1">
       <c r="A40" s="105"/>
       <c r="B40" s="172" t="str" cm="1">
         <f t="array" aca="1" ref="B40" ca="1">CONCATENATE("报价人：", INDIRECT("项目信息!$B$8"))</f>
@@ -4085,54 +5516,54 @@
       <c r="P40" s="4"/>
       <c r="Q40" s="4"/>
     </row>
-    <row r="41" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A41" s="174" t="str">
+    <row r="41" spans="1:21" ht="18" customHeight="1">
+      <c r="A41" s="287" t="str">
         <f ca="1">T(INDIRECT("项目信息!B22"))</f>
         <v>扬州华科</v>
       </c>
-      <c r="B41" s="174"/>
-      <c r="C41" s="174"/>
-      <c r="D41" s="174"/>
-      <c r="E41" s="174"/>
-      <c r="F41" s="174"/>
-      <c r="G41" s="174"/>
-      <c r="H41" s="174"/>
-      <c r="I41" s="174"/>
+      <c r="B41" s="287"/>
+      <c r="C41" s="287"/>
+      <c r="D41" s="287"/>
+      <c r="E41" s="287"/>
+      <c r="F41" s="287"/>
+      <c r="G41" s="287"/>
+      <c r="H41" s="287"/>
+      <c r="I41" s="287"/>
       <c r="Q41" s="1"/>
       <c r="R41" s="1"/>
     </row>
-    <row r="42" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A42" s="174" t="str">
+    <row r="42" spans="1:21" ht="18" customHeight="1">
+      <c r="A42" s="287" t="str">
         <f ca="1">T(INDIRECT("项目信息!B23"))</f>
         <v/>
       </c>
-      <c r="B42" s="174"/>
-      <c r="C42" s="174"/>
-      <c r="D42" s="174"/>
-      <c r="E42" s="174"/>
-      <c r="F42" s="174"/>
-      <c r="G42" s="174"/>
-      <c r="H42" s="174"/>
-      <c r="I42" s="174"/>
+      <c r="B42" s="287"/>
+      <c r="C42" s="287"/>
+      <c r="D42" s="287"/>
+      <c r="E42" s="287"/>
+      <c r="F42" s="287"/>
+      <c r="G42" s="287"/>
+      <c r="H42" s="287"/>
+      <c r="I42" s="287"/>
       <c r="Q42" s="1"/>
       <c r="R42" s="1"/>
     </row>
-    <row r="43" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A43" s="193" t="s">
+    <row r="43" spans="1:21" ht="18" customHeight="1">
+      <c r="A43" s="304" t="s">
         <v>64</v>
       </c>
-      <c r="B43" s="193"/>
-      <c r="C43" s="193"/>
-      <c r="D43" s="193"/>
-      <c r="E43" s="193"/>
-      <c r="F43" s="193"/>
-      <c r="G43" s="193"/>
-      <c r="H43" s="193"/>
-      <c r="I43" s="193"/>
+      <c r="B43" s="304"/>
+      <c r="C43" s="304"/>
+      <c r="D43" s="304"/>
+      <c r="E43" s="304"/>
+      <c r="F43" s="304"/>
+      <c r="G43" s="304"/>
+      <c r="H43" s="304"/>
+      <c r="I43" s="304"/>
       <c r="Q43" s="1"/>
       <c r="R43" s="1"/>
     </row>
-    <row r="44" spans="1:21" s="127" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="44" spans="1:21" s="127" customFormat="1" ht="18" customHeight="1">
       <c r="A44" s="119" t="s">
         <v>92</v>
       </c>
@@ -4142,17 +5573,17 @@
       <c r="C44" s="121" t="s">
         <v>65</v>
       </c>
-      <c r="D44" s="173" t="s">
-        <v>8</v>
-      </c>
-      <c r="E44" s="173"/>
+      <c r="D44" s="286" t="s">
+        <v>8</v>
+      </c>
+      <c r="E44" s="286"/>
       <c r="F44" s="122" t="s">
         <v>66</v>
       </c>
-      <c r="G44" s="173" t="s">
-        <v>8</v>
-      </c>
-      <c r="H44" s="173"/>
+      <c r="G44" s="286" t="s">
+        <v>8</v>
+      </c>
+      <c r="H44" s="286"/>
       <c r="I44" s="123" t="s">
         <v>8</v>
       </c>
@@ -4174,7 +5605,7 @@
       <c r="Q44" s="5"/>
       <c r="R44" s="5"/>
     </row>
-    <row r="45" spans="1:21" s="4" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:21" s="4" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A45" s="15" t="s">
         <v>29</v>
       </c>
@@ -4239,7 +5670,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="46" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="46" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A46" s="64">
         <f t="shared" ref="A46:A70" si="1">ROW()-ROW(A$45)</f>
         <v>1</v>
@@ -4307,7 +5738,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="47" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A47" s="46">
         <f t="shared" si="1"/>
         <v>2</v>
@@ -4375,7 +5806,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="48" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="48" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A48" s="46">
         <f t="shared" si="1"/>
         <v>3</v>
@@ -4443,7 +5874,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="49" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="49" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A49" s="46">
         <f t="shared" si="1"/>
         <v>4</v>
@@ -4511,7 +5942,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="50" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="50" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A50" s="46">
         <f t="shared" si="1"/>
         <v>5</v>
@@ -4579,7 +6010,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="51" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="51" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A51" s="46">
         <f t="shared" si="1"/>
         <v>6</v>
@@ -4647,7 +6078,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="52" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="52" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A52" s="46">
         <f t="shared" si="1"/>
         <v>7</v>
@@ -4715,7 +6146,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="53" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="53" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A53" s="46">
         <f t="shared" si="1"/>
         <v>8</v>
@@ -4783,7 +6214,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="54" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="54" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A54" s="46">
         <f t="shared" si="1"/>
         <v>9</v>
@@ -4851,7 +6282,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="55" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="55" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A55" s="46">
         <f t="shared" si="1"/>
         <v>10</v>
@@ -4919,7 +6350,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="56" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="56" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A56" s="46">
         <f t="shared" si="1"/>
         <v>11</v>
@@ -4987,7 +6418,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="57" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="57" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A57" s="46">
         <f t="shared" si="1"/>
         <v>12</v>
@@ -5055,7 +6486,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="58" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="58" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A58" s="46">
         <f t="shared" si="1"/>
         <v>13</v>
@@ -5123,7 +6554,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="59" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="59" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A59" s="46">
         <f t="shared" si="1"/>
         <v>14</v>
@@ -5191,7 +6622,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="60" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="60" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A60" s="46">
         <f t="shared" si="1"/>
         <v>15</v>
@@ -5259,7 +6690,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="61" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="61" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A61" s="46">
         <f t="shared" si="1"/>
         <v>16</v>
@@ -5327,7 +6758,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="62" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="62" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A62" s="46">
         <f t="shared" si="1"/>
         <v>17</v>
@@ -5395,7 +6826,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="63" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="63" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A63" s="46">
         <f t="shared" si="1"/>
         <v>18</v>
@@ -5463,7 +6894,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="64" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="64" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A64" s="46">
         <f t="shared" si="1"/>
         <v>19</v>
@@ -5531,7 +6962,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="65" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="65" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A65" s="46">
         <f t="shared" si="1"/>
         <v>20</v>
@@ -5599,7 +7030,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="66" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="66" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A66" s="46">
         <f t="shared" si="1"/>
         <v>21</v>
@@ -5645,7 +7076,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="67" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="67" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A67" s="46">
         <f t="shared" si="1"/>
         <v>22</v>
@@ -5687,7 +7118,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="68" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="68" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A68" s="46">
         <f t="shared" si="1"/>
         <v>23</v>
@@ -5724,7 +7155,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="69" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="69" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A69" s="46">
         <f t="shared" si="1"/>
         <v>24</v>
@@ -5763,7 +7194,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="70" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="70" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A70" s="46">
         <f t="shared" si="1"/>
         <v>25</v>
@@ -5801,7 +7232,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="71" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="71" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="A71" s="150" t="s">
         <v>87</v>
       </c>
@@ -5843,7 +7274,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="72" spans="1:21" s="127" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="72" spans="1:21" s="127" customFormat="1" ht="18" customHeight="1">
       <c r="A72" s="103"/>
       <c r="B72" s="125" t="s">
         <v>8</v>
@@ -5860,7 +7291,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="73" spans="1:21" s="127" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="73" spans="1:21" s="127" customFormat="1" ht="18" customHeight="1">
       <c r="A73" s="103"/>
       <c r="B73" s="125" t="s">
         <v>8</v>
@@ -5877,7 +7308,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="74" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="74" spans="1:21" s="4" customFormat="1" ht="18" customHeight="1">
       <c r="B74" s="172" t="str" cm="1">
         <f t="array" aca="1" ref="B74" ca="1">CONCATENATE("报价人：", INDIRECT("项目信息!$B$8"))</f>
         <v>报价人：李四</v>
@@ -5897,7 +7328,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="75" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="75" spans="1:21" ht="18" customHeight="1">
       <c r="A75" s="158"/>
     </row>
   </sheetData>
@@ -5939,4 +7370,741 @@
   </customProperties>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8843F8F8-878A-4798-8AFC-517D2311E176}">
+  <dimension ref="A1:AC12"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="4.375" style="224" customWidth="1"/>
+    <col min="2" max="2" width="14.875" style="224" customWidth="1"/>
+    <col min="3" max="3" width="34.625" style="224" customWidth="1"/>
+    <col min="4" max="4" width="5.375" style="224" customWidth="1"/>
+    <col min="5" max="5" width="5" style="224" customWidth="1"/>
+    <col min="6" max="6" width="15.625" style="224" customWidth="1"/>
+    <col min="7" max="7" width="10.5" style="228" customWidth="1"/>
+    <col min="8" max="8" width="11.75" style="229" customWidth="1"/>
+    <col min="9" max="10" width="8.75" style="224" customWidth="1"/>
+    <col min="11" max="14" width="8.75" style="225" customWidth="1"/>
+    <col min="15" max="18" width="9" style="199" customWidth="1"/>
+    <col min="19" max="26" width="9" style="200"/>
+    <col min="27" max="27" width="9" style="201"/>
+    <col min="28" max="29" width="9" style="202" hidden="1" customWidth="1"/>
+    <col min="30" max="16384" width="9" style="203"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:29" ht="47.25" customHeight="1">
+      <c r="A1" s="230" t="s">
+        <v>126</v>
+      </c>
+      <c r="B1" s="195"/>
+      <c r="C1" s="195"/>
+      <c r="D1" s="195"/>
+      <c r="E1" s="195"/>
+      <c r="F1" s="195"/>
+      <c r="G1" s="195"/>
+      <c r="H1" s="196"/>
+      <c r="I1" s="195"/>
+      <c r="J1" s="197"/>
+      <c r="K1" s="198"/>
+      <c r="L1" s="198"/>
+      <c r="M1" s="198"/>
+      <c r="N1" s="198"/>
+    </row>
+    <row r="2" spans="1:29" ht="30" customHeight="1">
+      <c r="A2" s="204" t="s">
+        <v>125</v>
+      </c>
+      <c r="B2" s="204"/>
+      <c r="C2" s="204"/>
+      <c r="D2" s="204"/>
+      <c r="E2" s="204"/>
+      <c r="F2" s="204"/>
+      <c r="G2" s="204"/>
+      <c r="H2" s="205"/>
+      <c r="I2" s="204"/>
+      <c r="J2" s="206"/>
+      <c r="K2" s="207"/>
+      <c r="L2" s="207"/>
+      <c r="M2" s="207"/>
+      <c r="N2" s="207"/>
+    </row>
+    <row r="3" spans="1:29" ht="12" customHeight="1">
+      <c r="A3" s="208"/>
+      <c r="B3" s="208"/>
+      <c r="C3" s="208"/>
+      <c r="D3" s="208"/>
+      <c r="E3" s="208"/>
+      <c r="F3" s="208"/>
+      <c r="G3" s="209"/>
+      <c r="H3" s="210"/>
+      <c r="I3" s="208"/>
+      <c r="J3" s="211"/>
+      <c r="K3" s="212"/>
+      <c r="L3" s="212"/>
+      <c r="M3" s="212"/>
+      <c r="N3" s="212"/>
+    </row>
+    <row r="4" spans="1:29" s="220" customFormat="1">
+      <c r="A4" s="213" t="s">
+        <v>127</v>
+      </c>
+      <c r="B4" s="213"/>
+      <c r="C4" s="214"/>
+      <c r="D4" s="214"/>
+      <c r="E4" s="213"/>
+      <c r="F4" s="213"/>
+      <c r="G4" s="213"/>
+      <c r="H4" s="215"/>
+      <c r="I4" s="213"/>
+      <c r="J4" s="216"/>
+      <c r="K4" s="217"/>
+      <c r="L4" s="217"/>
+      <c r="M4" s="217"/>
+      <c r="N4" s="217"/>
+      <c r="O4" s="217"/>
+      <c r="P4" s="217"/>
+      <c r="Q4" s="217"/>
+      <c r="R4" s="217"/>
+      <c r="S4" s="216"/>
+      <c r="T4" s="216"/>
+      <c r="U4" s="216"/>
+      <c r="V4" s="216"/>
+      <c r="W4" s="216"/>
+      <c r="X4" s="216"/>
+      <c r="Y4" s="216"/>
+      <c r="Z4" s="216"/>
+      <c r="AA4" s="218"/>
+      <c r="AB4" s="219"/>
+      <c r="AC4" s="219"/>
+    </row>
+    <row r="5" spans="1:29" customFormat="1" ht="16.899999999999999" customHeight="1">
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+    </row>
+    <row r="6" spans="1:29" ht="16.899999999999999" customHeight="1">
+      <c r="A6" s="221" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="221" t="s">
+        <v>119</v>
+      </c>
+      <c r="C6" s="221" t="s">
+        <v>120</v>
+      </c>
+      <c r="D6" s="221" t="s">
+        <v>46</v>
+      </c>
+      <c r="E6" s="221" t="s">
+        <v>121</v>
+      </c>
+      <c r="F6" s="221" t="s">
+        <v>122</v>
+      </c>
+      <c r="G6" s="222" t="s">
+        <v>123</v>
+      </c>
+      <c r="H6" s="223" t="s">
+        <v>124</v>
+      </c>
+      <c r="I6" s="221" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:29" ht="24.95" customHeight="1">
+      <c r="A7" s="226"/>
+      <c r="B7" s="226" t="s">
+        <v>128</v>
+      </c>
+      <c r="C7" s="226" t="s">
+        <v>129</v>
+      </c>
+      <c r="D7" s="226" t="s">
+        <v>130</v>
+      </c>
+      <c r="E7" s="226" t="s">
+        <v>131</v>
+      </c>
+      <c r="F7" s="226"/>
+      <c r="G7" s="227"/>
+      <c r="H7" s="227"/>
+      <c r="I7" s="226" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="8" spans="1:29" ht="24.95" customHeight="1">
+      <c r="A8" s="226"/>
+      <c r="B8" s="226"/>
+      <c r="C8" s="226"/>
+      <c r="D8" s="226"/>
+      <c r="E8" s="226"/>
+      <c r="F8" s="226"/>
+      <c r="G8" s="227"/>
+      <c r="H8" s="227"/>
+      <c r="I8" s="226"/>
+    </row>
+    <row r="9" spans="1:29" ht="24.95" customHeight="1">
+      <c r="A9" s="226"/>
+      <c r="B9" s="226"/>
+      <c r="C9" s="226"/>
+      <c r="D9" s="226"/>
+      <c r="E9" s="226"/>
+      <c r="F9" s="226"/>
+      <c r="G9" s="227"/>
+      <c r="H9" s="227"/>
+      <c r="I9" s="226"/>
+    </row>
+    <row r="10" spans="1:29" ht="24.95" customHeight="1">
+      <c r="A10" s="226"/>
+      <c r="B10" s="226"/>
+      <c r="C10" s="226"/>
+      <c r="D10" s="226"/>
+      <c r="E10" s="226"/>
+      <c r="F10" s="226"/>
+      <c r="G10" s="227"/>
+      <c r="H10" s="227"/>
+      <c r="I10" s="226"/>
+    </row>
+    <row r="11" spans="1:29" ht="24.95" customHeight="1">
+      <c r="A11" s="226"/>
+      <c r="B11" s="226"/>
+      <c r="C11" s="226"/>
+      <c r="D11" s="226"/>
+      <c r="E11" s="226"/>
+      <c r="F11" s="226"/>
+      <c r="G11" s="227"/>
+      <c r="H11" s="227"/>
+      <c r="I11" s="226"/>
+    </row>
+    <row r="12" spans="1:29" ht="24.95" customHeight="1">
+      <c r="A12" s="226"/>
+      <c r="B12" s="226"/>
+      <c r="C12" s="226"/>
+      <c r="D12" s="226"/>
+      <c r="E12" s="226"/>
+      <c r="F12" s="226"/>
+      <c r="G12" s="227"/>
+      <c r="H12" s="227"/>
+      <c r="I12" s="226"/>
+    </row>
+  </sheetData>
+  <dataConsolidate/>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.98425196850393704" bottom="0.98425196850393704" header="0.51181102362204722" footer="0.51181102362204722"/>
+  <pageSetup paperSize="9" scale="97" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <headerFooter alignWithMargins="0">
+    <oddFooter>第 &amp;P 页，共 &amp;N 页</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93EB2E83-8D75-45D5-99A4-19975F907CE1}">
+  <dimension ref="A1:H31"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="5.5" style="203" customWidth="1"/>
+    <col min="2" max="2" width="9.125" style="203" customWidth="1"/>
+    <col min="3" max="3" width="23.25" style="231" customWidth="1"/>
+    <col min="4" max="5" width="7.5" style="203" customWidth="1"/>
+    <col min="6" max="6" width="12.625" style="232" customWidth="1"/>
+    <col min="7" max="7" width="16.375" style="232" customWidth="1"/>
+    <col min="8" max="8" width="14.625" style="203" customWidth="1"/>
+    <col min="9" max="16384" width="9" style="203"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="203" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="31.5">
+      <c r="A2" s="248" t="s">
+        <v>157</v>
+      </c>
+      <c r="B2" s="248"/>
+      <c r="C2" s="248"/>
+      <c r="D2" s="248"/>
+      <c r="E2" s="248"/>
+      <c r="F2" s="248"/>
+      <c r="G2" s="248"/>
+    </row>
+    <row r="3" spans="1:8" ht="31.5">
+      <c r="A3" s="248" t="s">
+        <v>134</v>
+      </c>
+      <c r="B3" s="248"/>
+      <c r="C3" s="248"/>
+      <c r="D3" s="248"/>
+      <c r="E3" s="248"/>
+      <c r="F3" s="248"/>
+      <c r="G3" s="248"/>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="233" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" s="231"/>
+      <c r="D4" s="231"/>
+      <c r="E4" s="231"/>
+      <c r="F4" s="234"/>
+      <c r="G4" s="234"/>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="249" t="s">
+        <v>146</v>
+      </c>
+      <c r="B5" s="249"/>
+      <c r="C5" s="249"/>
+      <c r="D5" s="249"/>
+      <c r="E5" s="249"/>
+      <c r="F5" s="249"/>
+      <c r="G5" s="249"/>
+    </row>
+    <row r="6" spans="1:8" ht="20.100000000000001" customHeight="1">
+      <c r="A6" s="235" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="235" t="s">
+        <v>119</v>
+      </c>
+      <c r="C6" s="235" t="s">
+        <v>136</v>
+      </c>
+      <c r="D6" s="235" t="s">
+        <v>47</v>
+      </c>
+      <c r="E6" s="235" t="s">
+        <v>46</v>
+      </c>
+      <c r="F6" s="236" t="s">
+        <v>137</v>
+      </c>
+      <c r="G6" s="236" t="s">
+        <v>138</v>
+      </c>
+      <c r="H6" s="235" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="36.6" customHeight="1">
+      <c r="A7" s="237" t="s">
+        <v>147</v>
+      </c>
+      <c r="B7" s="235" t="s">
+        <v>148</v>
+      </c>
+      <c r="C7" s="238" t="s">
+        <v>149</v>
+      </c>
+      <c r="D7" s="235" t="s">
+        <v>131</v>
+      </c>
+      <c r="E7" s="235" t="s">
+        <v>97</v>
+      </c>
+      <c r="F7" s="236" t="s">
+        <v>150</v>
+      </c>
+      <c r="G7" s="236"/>
+      <c r="H7" s="235"/>
+    </row>
+    <row r="8" spans="1:8" ht="36.6" customHeight="1">
+      <c r="A8" s="237"/>
+      <c r="B8" s="235"/>
+      <c r="C8" s="238"/>
+      <c r="D8" s="235"/>
+      <c r="E8" s="235"/>
+      <c r="F8" s="236"/>
+      <c r="G8" s="236"/>
+      <c r="H8" s="235"/>
+    </row>
+    <row r="9" spans="1:8" ht="20.100000000000001" customHeight="1">
+      <c r="A9" s="237"/>
+      <c r="B9" s="235"/>
+      <c r="C9" s="238"/>
+      <c r="D9" s="235"/>
+      <c r="E9" s="235"/>
+      <c r="F9" s="236"/>
+      <c r="G9" s="236"/>
+      <c r="H9" s="235"/>
+    </row>
+    <row r="10" spans="1:8" ht="20.100000000000001" customHeight="1">
+      <c r="A10" s="239"/>
+      <c r="B10" s="240"/>
+      <c r="C10" s="240"/>
+      <c r="D10" s="240"/>
+      <c r="E10" s="240"/>
+      <c r="F10" s="241"/>
+      <c r="G10" s="241"/>
+      <c r="H10" s="240"/>
+    </row>
+    <row r="11" spans="1:8" ht="20.100000000000001" customHeight="1">
+      <c r="A11" s="239"/>
+      <c r="B11" s="240"/>
+      <c r="C11" s="240"/>
+      <c r="D11" s="240"/>
+      <c r="E11" s="240"/>
+      <c r="F11" s="241"/>
+      <c r="G11" s="241"/>
+      <c r="H11" s="240"/>
+    </row>
+    <row r="12" spans="1:8" ht="20.100000000000001" customHeight="1">
+      <c r="A12" s="239"/>
+      <c r="B12" s="240"/>
+      <c r="C12" s="240"/>
+      <c r="D12" s="240"/>
+      <c r="E12" s="240"/>
+      <c r="F12" s="241"/>
+      <c r="G12" s="241"/>
+      <c r="H12" s="240"/>
+    </row>
+    <row r="13" spans="1:8" ht="20.100000000000001" customHeight="1">
+      <c r="A13" s="242"/>
+      <c r="B13" s="242" t="s">
+        <v>140</v>
+      </c>
+      <c r="C13" s="242"/>
+      <c r="D13" s="242">
+        <f>SUM(D6:D12)</f>
+        <v>0</v>
+      </c>
+      <c r="E13" s="242" t="s">
+        <v>141</v>
+      </c>
+      <c r="F13" s="243"/>
+      <c r="G13" s="243">
+        <f>ROUND(SUM(G6:G12),0)</f>
+        <v>0</v>
+      </c>
+      <c r="H13" s="244"/>
+    </row>
+    <row r="14" spans="1:8" s="246" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="A14" s="305" t="str">
+        <f>"合计RMB："&amp; TEXT(SUBSTITUTE(IF(G13="","",IF(MOD(G13,1)=0,TEXT(INT(G13),"[DBNum2][$-804]G/通用格式元整"),(TEXT(INT(G13),"[DBNum2][$-804]G/通用格式元")&amp;TEXT((INT(G13*10)-INT(G13)*10),"[DBNum2][$-804]G/通用格式角")&amp;TEXT((INT(G13*100)-INT(G13*10)*10),"[DBNum2][$-804]G/通用格式分")))),"零角","零"),)</f>
+        <v>合计RMB：零元整</v>
+      </c>
+      <c r="B14" s="305"/>
+      <c r="C14" s="305"/>
+      <c r="D14" s="305"/>
+      <c r="E14" s="305"/>
+      <c r="F14" s="305"/>
+      <c r="G14" s="305"/>
+      <c r="H14" s="245"/>
+    </row>
+    <row r="15" spans="1:8" ht="20.100000000000001" customHeight="1"/>
+    <row r="16" spans="1:8" ht="20.100000000000001" customHeight="1">
+      <c r="A16" s="203" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="20.100000000000001" customHeight="1">
+      <c r="F17" s="231"/>
+      <c r="G17" s="203"/>
+    </row>
+    <row r="18" spans="1:7" ht="20.100000000000001" customHeight="1">
+      <c r="F18" s="247"/>
+      <c r="G18" s="247"/>
+    </row>
+    <row r="19" spans="1:7" ht="20.100000000000001" customHeight="1">
+      <c r="F19" s="203"/>
+      <c r="G19" s="203"/>
+    </row>
+    <row r="20" spans="1:7" ht="20.100000000000001" customHeight="1"/>
+    <row r="21" spans="1:7" ht="20.100000000000001" customHeight="1"/>
+    <row r="22" spans="1:7" ht="20.100000000000001" customHeight="1"/>
+    <row r="23" spans="1:7" ht="20.100000000000001" customHeight="1">
+      <c r="D23" s="231"/>
+    </row>
+    <row r="24" spans="1:7" ht="20.100000000000001" customHeight="1">
+      <c r="D24" s="231"/>
+    </row>
+    <row r="25" spans="1:7" ht="20.100000000000001" customHeight="1"/>
+    <row r="26" spans="1:7" ht="20.100000000000001" customHeight="1"/>
+    <row r="27" spans="1:7" ht="20.100000000000001" customHeight="1"/>
+    <row r="28" spans="1:7" ht="20.100000000000001" customHeight="1"/>
+    <row r="29" spans="1:7" s="231" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="A29" s="203"/>
+      <c r="B29" s="203"/>
+      <c r="D29" s="203"/>
+      <c r="E29" s="203"/>
+      <c r="F29" s="232"/>
+      <c r="G29" s="232"/>
+    </row>
+    <row r="30" spans="1:7" ht="20.100000000000001" customHeight="1"/>
+    <row r="31" spans="1:7" ht="20.100000000000001" customHeight="1"/>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A14:G14"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="90" orientation="portrait" r:id="rId1"/>
+  <headerFooter alignWithMargins="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3534982B-B631-4E68-8B11-E0B2E3DE60A9}">
+  <dimension ref="A1:J23"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="5.5" style="203" customWidth="1"/>
+    <col min="2" max="2" width="9.125" style="203" customWidth="1"/>
+    <col min="3" max="3" width="23.25" style="231" customWidth="1"/>
+    <col min="4" max="5" width="7.5" style="203" customWidth="1"/>
+    <col min="6" max="6" width="10.25" style="203" customWidth="1"/>
+    <col min="7" max="7" width="13.875" style="203" customWidth="1"/>
+    <col min="8" max="8" width="20.625" style="232" customWidth="1"/>
+    <col min="9" max="9" width="14.625" style="203" customWidth="1"/>
+    <col min="10" max="16384" width="9" style="203"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="203" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="31.5">
+      <c r="A2" s="248" t="s">
+        <v>157</v>
+      </c>
+      <c r="B2" s="248"/>
+      <c r="C2" s="248"/>
+      <c r="D2" s="248"/>
+      <c r="E2" s="248"/>
+      <c r="F2" s="248"/>
+      <c r="G2" s="248"/>
+      <c r="H2" s="248"/>
+      <c r="I2" s="231"/>
+    </row>
+    <row r="3" spans="1:9" ht="31.5">
+      <c r="A3" s="248" t="s">
+        <v>143</v>
+      </c>
+      <c r="B3" s="248"/>
+      <c r="C3" s="248"/>
+      <c r="D3" s="248"/>
+      <c r="E3" s="248"/>
+      <c r="F3" s="248"/>
+      <c r="G3" s="248"/>
+      <c r="H3" s="248"/>
+      <c r="I3" s="231"/>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="233" t="s">
+        <v>144</v>
+      </c>
+      <c r="B4" s="231"/>
+      <c r="D4" s="231"/>
+      <c r="E4" s="231"/>
+      <c r="F4" s="231"/>
+      <c r="G4" s="231"/>
+      <c r="H4" s="234"/>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="249" t="str">
+        <f>[1]报价明细!A4</f>
+        <v>项目名称：GZ460</v>
+      </c>
+      <c r="B5" s="249"/>
+      <c r="C5" s="249"/>
+      <c r="D5" s="249"/>
+      <c r="E5" s="249"/>
+      <c r="F5" s="249"/>
+      <c r="G5" s="249"/>
+      <c r="H5" s="249"/>
+    </row>
+    <row r="6" spans="1:9" ht="20.100000000000001" customHeight="1">
+      <c r="A6" s="235" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="235" t="s">
+        <v>119</v>
+      </c>
+      <c r="C6" s="235" t="s">
+        <v>136</v>
+      </c>
+      <c r="D6" s="235" t="s">
+        <v>47</v>
+      </c>
+      <c r="E6" s="235" t="s">
+        <v>46</v>
+      </c>
+      <c r="F6" s="235" t="s">
+        <v>153</v>
+      </c>
+      <c r="G6" s="235" t="s">
+        <v>151</v>
+      </c>
+      <c r="H6" s="236" t="s">
+        <v>152</v>
+      </c>
+      <c r="I6" s="235" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="36.6" customHeight="1">
+      <c r="A7" s="237" t="s">
+        <v>147</v>
+      </c>
+      <c r="B7" s="235" t="s">
+        <v>139</v>
+      </c>
+      <c r="C7" s="238" t="s">
+        <v>149</v>
+      </c>
+      <c r="D7" s="235" t="s">
+        <v>131</v>
+      </c>
+      <c r="E7" s="235" t="s">
+        <v>97</v>
+      </c>
+      <c r="F7" s="235" t="s">
+        <v>154</v>
+      </c>
+      <c r="G7" s="235" t="s">
+        <v>155</v>
+      </c>
+      <c r="H7" s="236"/>
+      <c r="I7" s="235" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="36.6" customHeight="1">
+      <c r="A8" s="237"/>
+      <c r="B8" s="235"/>
+      <c r="C8" s="238"/>
+      <c r="D8" s="235"/>
+      <c r="E8" s="235"/>
+      <c r="F8" s="235"/>
+      <c r="G8" s="235"/>
+      <c r="H8" s="236"/>
+      <c r="I8" s="235"/>
+    </row>
+    <row r="9" spans="1:9" ht="20.100000000000001" customHeight="1">
+      <c r="A9" s="237"/>
+      <c r="B9" s="235"/>
+      <c r="C9" s="238"/>
+      <c r="D9" s="235"/>
+      <c r="E9" s="235"/>
+      <c r="F9" s="235"/>
+      <c r="G9" s="235"/>
+      <c r="H9" s="236"/>
+      <c r="I9" s="235"/>
+    </row>
+    <row r="10" spans="1:9" ht="20.100000000000001" customHeight="1">
+      <c r="A10" s="239"/>
+      <c r="B10" s="240"/>
+      <c r="C10" s="240"/>
+      <c r="D10" s="240"/>
+      <c r="E10" s="240"/>
+      <c r="F10" s="240"/>
+      <c r="G10" s="240"/>
+      <c r="H10" s="241"/>
+      <c r="I10" s="240"/>
+    </row>
+    <row r="11" spans="1:9" ht="20.100000000000001" customHeight="1">
+      <c r="A11" s="239"/>
+      <c r="B11" s="240"/>
+      <c r="C11" s="240"/>
+      <c r="D11" s="240"/>
+      <c r="E11" s="240"/>
+      <c r="F11" s="240"/>
+      <c r="G11" s="240"/>
+      <c r="H11" s="241"/>
+      <c r="I11" s="240"/>
+    </row>
+    <row r="12" spans="1:9" ht="20.100000000000001" customHeight="1">
+      <c r="A12" s="239"/>
+      <c r="B12" s="240"/>
+      <c r="C12" s="240"/>
+      <c r="D12" s="240"/>
+      <c r="E12" s="240"/>
+      <c r="F12" s="240"/>
+      <c r="G12" s="240"/>
+      <c r="H12" s="241"/>
+      <c r="I12" s="240"/>
+    </row>
+    <row r="13" spans="1:9" ht="20.100000000000001" customHeight="1">
+      <c r="A13" s="242"/>
+      <c r="B13" s="242" t="s">
+        <v>140</v>
+      </c>
+      <c r="C13" s="242"/>
+      <c r="D13" s="242">
+        <f>SUM(D6:D12)</f>
+        <v>0</v>
+      </c>
+      <c r="E13" s="242" t="s">
+        <v>141</v>
+      </c>
+      <c r="F13" s="242"/>
+      <c r="G13" s="242"/>
+      <c r="H13" s="243">
+        <f>ROUND(SUM(H6:H12),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I13" s="244"/>
+    </row>
+    <row r="14" spans="1:9" ht="20.100000000000001" customHeight="1"/>
+    <row r="15" spans="1:9" ht="20.100000000000001" customHeight="1">
+      <c r="A15" s="203" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="20.100000000000001" customHeight="1">
+      <c r="H16" s="203"/>
+    </row>
+    <row r="17" spans="1:10" ht="20.100000000000001" customHeight="1"/>
+    <row r="18" spans="1:10" ht="20.100000000000001" customHeight="1">
+      <c r="C18" s="203"/>
+      <c r="E18" s="231"/>
+      <c r="F18" s="231"/>
+      <c r="G18" s="231"/>
+      <c r="H18" s="203"/>
+      <c r="J18" s="232"/>
+    </row>
+    <row r="19" spans="1:10" ht="20.100000000000001" customHeight="1">
+      <c r="C19" s="203"/>
+      <c r="E19" s="231"/>
+      <c r="F19" s="231"/>
+      <c r="G19" s="231"/>
+      <c r="H19" s="203"/>
+      <c r="J19" s="232"/>
+    </row>
+    <row r="20" spans="1:10" ht="20.100000000000001" customHeight="1">
+      <c r="C20" s="203"/>
+      <c r="E20" s="231"/>
+      <c r="F20" s="231"/>
+      <c r="G20" s="231"/>
+      <c r="H20" s="203"/>
+      <c r="J20" s="232"/>
+    </row>
+    <row r="21" spans="1:10" s="231" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="A21" s="203"/>
+      <c r="B21" s="203"/>
+      <c r="D21" s="203"/>
+      <c r="E21" s="203"/>
+      <c r="F21" s="203"/>
+      <c r="G21" s="203"/>
+      <c r="H21" s="232"/>
+    </row>
+    <row r="22" spans="1:10" ht="20.100000000000001" customHeight="1"/>
+    <row r="23" spans="1:10" ht="20.100000000000001" customHeight="1"/>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A5:H5"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="90" orientation="portrait" r:id="rId1"/>
+  <headerFooter alignWithMargins="0"/>
+</worksheet>
 </file>
</xml_diff>